<commit_message>
Mise à jour du modèle de planning pour Lundi et Mardi
</commit_message>
<xml_diff>
--- a/documentation/3_2_Modele_PlanningLundiMardi.xlsx
+++ b/documentation/3_2_Modele_PlanningLundiMardi.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eloua\Documents\projet-306-tercier-morales-bersier\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E05747F-F3B8-4ED8-A122-591C88C662CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6630A76D-76C9-46A4-8963-6FC9C10F79DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Planning!$A:$C,Planning!$1:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Planning!$A$1:$CE$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Planning!$A$1:$CE$46</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="64">
   <si>
     <t>Tous</t>
   </si>
@@ -495,6 +495,12 @@
   <si>
     <t>1+AZ8:AZ38</t>
   </si>
+  <si>
+    <t>débugage</t>
+  </si>
+  <si>
+    <t>création de la démo</t>
+  </si>
 </sst>
 </file>
 
@@ -717,7 +723,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -1071,12 +1077,58 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -1279,6 +1331,86 @@
     <xf numFmtId="0" fontId="3" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" textRotation="90"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -1291,30 +1423,6 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1323,60 +1431,39 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" textRotation="90"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1432,7 +1519,7 @@
     <xdr:to>
       <xdr:col>88</xdr:col>
       <xdr:colOff>231855</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>56546</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1858,7 +1945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CF45"/>
+  <dimension ref="A1:CF47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="66.7265625" style="3" customWidth="1"/>
@@ -1871,11 +1958,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:84" ht="23" x14ac:dyDescent="0.5">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="79" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
       <c r="D1" s="1" t="s">
         <v>38</v>
       </c>
@@ -1923,8 +2010,8 @@
       <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
+      <c r="B2" s="82"/>
+      <c r="C2" s="82"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -2017,8 +2104,8 @@
       <c r="A4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
+      <c r="B4" s="83"/>
+      <c r="C4" s="83"/>
       <c r="D4" s="1" t="s">
         <v>15</v>
       </c>
@@ -2069,90 +2156,90 @@
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="60"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="66">
+      <c r="B5" s="80"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="77">
         <v>0</v>
       </c>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
-      <c r="H5" s="66"/>
-      <c r="I5" s="66"/>
-      <c r="J5" s="66"/>
-      <c r="K5" s="66"/>
-      <c r="L5" s="66"/>
-      <c r="M5" s="66"/>
-      <c r="N5" s="66"/>
-      <c r="O5" s="66"/>
-      <c r="P5" s="66"/>
-      <c r="Q5" s="66"/>
-      <c r="R5" s="66"/>
-      <c r="S5" s="66"/>
-      <c r="T5" s="66"/>
-      <c r="U5" s="66"/>
-      <c r="V5" s="66"/>
-      <c r="W5" s="66"/>
-      <c r="X5" s="66"/>
-      <c r="Y5" s="66"/>
-      <c r="Z5" s="66"/>
-      <c r="AA5" s="66"/>
-      <c r="AB5" s="66"/>
-      <c r="AC5" s="66"/>
-      <c r="AD5" s="66"/>
-      <c r="AE5" s="66"/>
-      <c r="AF5" s="66"/>
-      <c r="AG5" s="66"/>
-      <c r="AH5" s="66"/>
-      <c r="AI5" s="66"/>
-      <c r="AJ5" s="66"/>
-      <c r="AK5" s="66"/>
-      <c r="AL5" s="66"/>
-      <c r="AM5" s="66"/>
-      <c r="AN5" s="66"/>
-      <c r="AO5" s="66"/>
-      <c r="AP5" s="66"/>
-      <c r="AQ5" s="66"/>
-      <c r="AR5" s="66"/>
-      <c r="AS5" s="66"/>
-      <c r="AT5" s="66"/>
-      <c r="AU5" s="66"/>
-      <c r="AV5" s="66"/>
-      <c r="AW5" s="66"/>
-      <c r="AX5" s="66"/>
-      <c r="AY5" s="66"/>
-      <c r="AZ5" s="66"/>
-      <c r="BA5" s="66"/>
-      <c r="BB5" s="66"/>
-      <c r="BC5" s="66"/>
-      <c r="BD5" s="66"/>
-      <c r="BE5" s="66"/>
-      <c r="BF5" s="66"/>
-      <c r="BG5" s="66"/>
-      <c r="BH5" s="66"/>
-      <c r="BI5" s="66"/>
-      <c r="BJ5" s="66"/>
-      <c r="BK5" s="66"/>
-      <c r="BL5" s="66"/>
-      <c r="BM5" s="66"/>
-      <c r="BN5" s="66"/>
-      <c r="BO5" s="66"/>
-      <c r="BP5" s="66"/>
-      <c r="BQ5" s="66"/>
-      <c r="BR5" s="66"/>
-      <c r="BS5" s="66"/>
-      <c r="BT5" s="66"/>
-      <c r="BU5" s="66"/>
-      <c r="BV5" s="66"/>
-      <c r="BW5" s="66"/>
-      <c r="BX5" s="66"/>
-      <c r="BY5" s="66"/>
-      <c r="BZ5" s="66"/>
-      <c r="CA5" s="66"/>
-      <c r="CB5" s="66"/>
-      <c r="CC5" s="66"/>
-      <c r="CD5" s="66"/>
-      <c r="CE5" s="66"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="77"/>
+      <c r="J5" s="77"/>
+      <c r="K5" s="77"/>
+      <c r="L5" s="77"/>
+      <c r="M5" s="77"/>
+      <c r="N5" s="77"/>
+      <c r="O5" s="77"/>
+      <c r="P5" s="77"/>
+      <c r="Q5" s="77"/>
+      <c r="R5" s="77"/>
+      <c r="S5" s="77"/>
+      <c r="T5" s="77"/>
+      <c r="U5" s="77"/>
+      <c r="V5" s="77"/>
+      <c r="W5" s="77"/>
+      <c r="X5" s="77"/>
+      <c r="Y5" s="77"/>
+      <c r="Z5" s="77"/>
+      <c r="AA5" s="77"/>
+      <c r="AB5" s="77"/>
+      <c r="AC5" s="77"/>
+      <c r="AD5" s="77"/>
+      <c r="AE5" s="77"/>
+      <c r="AF5" s="77"/>
+      <c r="AG5" s="77"/>
+      <c r="AH5" s="77"/>
+      <c r="AI5" s="77"/>
+      <c r="AJ5" s="77"/>
+      <c r="AK5" s="77"/>
+      <c r="AL5" s="77"/>
+      <c r="AM5" s="77"/>
+      <c r="AN5" s="77"/>
+      <c r="AO5" s="77"/>
+      <c r="AP5" s="77"/>
+      <c r="AQ5" s="77"/>
+      <c r="AR5" s="77"/>
+      <c r="AS5" s="77"/>
+      <c r="AT5" s="77"/>
+      <c r="AU5" s="77"/>
+      <c r="AV5" s="77"/>
+      <c r="AW5" s="77"/>
+      <c r="AX5" s="77"/>
+      <c r="AY5" s="77"/>
+      <c r="AZ5" s="77"/>
+      <c r="BA5" s="77"/>
+      <c r="BB5" s="77"/>
+      <c r="BC5" s="77"/>
+      <c r="BD5" s="77"/>
+      <c r="BE5" s="77"/>
+      <c r="BF5" s="77"/>
+      <c r="BG5" s="77"/>
+      <c r="BH5" s="77"/>
+      <c r="BI5" s="77"/>
+      <c r="BJ5" s="77"/>
+      <c r="BK5" s="77"/>
+      <c r="BL5" s="77"/>
+      <c r="BM5" s="77"/>
+      <c r="BN5" s="77"/>
+      <c r="BO5" s="77"/>
+      <c r="BP5" s="77"/>
+      <c r="BQ5" s="77"/>
+      <c r="BR5" s="77"/>
+      <c r="BS5" s="77"/>
+      <c r="BT5" s="77"/>
+      <c r="BU5" s="77"/>
+      <c r="BV5" s="77"/>
+      <c r="BW5" s="77"/>
+      <c r="BX5" s="77"/>
+      <c r="BY5" s="77"/>
+      <c r="BZ5" s="77"/>
+      <c r="CA5" s="77"/>
+      <c r="CB5" s="77"/>
+      <c r="CC5" s="77"/>
+      <c r="CD5" s="77"/>
+      <c r="CE5" s="77"/>
     </row>
     <row r="6" spans="1:84" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
@@ -2160,89 +2247,89 @@
       </c>
       <c r="B6" s="26"/>
       <c r="C6" s="26"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
-      <c r="H6" s="67"/>
-      <c r="I6" s="67"/>
-      <c r="J6" s="67"/>
-      <c r="K6" s="67"/>
-      <c r="L6" s="67"/>
-      <c r="M6" s="67"/>
-      <c r="N6" s="67"/>
-      <c r="O6" s="67"/>
-      <c r="P6" s="67"/>
-      <c r="Q6" s="67"/>
-      <c r="R6" s="67"/>
-      <c r="S6" s="67"/>
-      <c r="T6" s="67"/>
-      <c r="U6" s="67"/>
-      <c r="V6" s="67"/>
-      <c r="W6" s="67"/>
-      <c r="X6" s="67"/>
-      <c r="Y6" s="67"/>
-      <c r="Z6" s="67"/>
-      <c r="AA6" s="67"/>
-      <c r="AB6" s="67"/>
-      <c r="AC6" s="67"/>
-      <c r="AD6" s="67"/>
-      <c r="AE6" s="67"/>
-      <c r="AF6" s="67"/>
-      <c r="AG6" s="67"/>
-      <c r="AH6" s="67"/>
-      <c r="AI6" s="67"/>
-      <c r="AJ6" s="67"/>
-      <c r="AK6" s="67"/>
-      <c r="AL6" s="67"/>
-      <c r="AM6" s="67"/>
-      <c r="AN6" s="67"/>
-      <c r="AO6" s="67"/>
-      <c r="AP6" s="67"/>
-      <c r="AQ6" s="67"/>
-      <c r="AR6" s="67"/>
-      <c r="AS6" s="67"/>
-      <c r="AT6" s="67"/>
-      <c r="AU6" s="67"/>
-      <c r="AV6" s="67"/>
-      <c r="AW6" s="67"/>
-      <c r="AX6" s="67"/>
-      <c r="AY6" s="67"/>
-      <c r="AZ6" s="67"/>
-      <c r="BA6" s="67"/>
-      <c r="BB6" s="67"/>
-      <c r="BC6" s="67"/>
-      <c r="BD6" s="67"/>
-      <c r="BE6" s="67"/>
-      <c r="BF6" s="67"/>
-      <c r="BG6" s="67"/>
-      <c r="BH6" s="67"/>
-      <c r="BI6" s="67"/>
-      <c r="BJ6" s="67"/>
-      <c r="BK6" s="67"/>
-      <c r="BL6" s="67"/>
-      <c r="BM6" s="67"/>
-      <c r="BN6" s="67"/>
-      <c r="BO6" s="67"/>
-      <c r="BP6" s="67"/>
-      <c r="BQ6" s="67"/>
-      <c r="BR6" s="67"/>
-      <c r="BS6" s="67"/>
-      <c r="BT6" s="67"/>
-      <c r="BU6" s="67"/>
-      <c r="BV6" s="67"/>
-      <c r="BW6" s="67"/>
-      <c r="BX6" s="67"/>
-      <c r="BY6" s="67"/>
-      <c r="BZ6" s="67"/>
-      <c r="CA6" s="67"/>
-      <c r="CB6" s="67"/>
-      <c r="CC6" s="67"/>
-      <c r="CD6" s="67"/>
-      <c r="CE6" s="67"/>
+      <c r="D6" s="78"/>
+      <c r="E6" s="78"/>
+      <c r="F6" s="78"/>
+      <c r="G6" s="78"/>
+      <c r="H6" s="78"/>
+      <c r="I6" s="78"/>
+      <c r="J6" s="78"/>
+      <c r="K6" s="78"/>
+      <c r="L6" s="78"/>
+      <c r="M6" s="78"/>
+      <c r="N6" s="78"/>
+      <c r="O6" s="78"/>
+      <c r="P6" s="78"/>
+      <c r="Q6" s="78"/>
+      <c r="R6" s="78"/>
+      <c r="S6" s="78"/>
+      <c r="T6" s="78"/>
+      <c r="U6" s="78"/>
+      <c r="V6" s="78"/>
+      <c r="W6" s="78"/>
+      <c r="X6" s="78"/>
+      <c r="Y6" s="78"/>
+      <c r="Z6" s="78"/>
+      <c r="AA6" s="78"/>
+      <c r="AB6" s="78"/>
+      <c r="AC6" s="78"/>
+      <c r="AD6" s="78"/>
+      <c r="AE6" s="78"/>
+      <c r="AF6" s="78"/>
+      <c r="AG6" s="78"/>
+      <c r="AH6" s="78"/>
+      <c r="AI6" s="78"/>
+      <c r="AJ6" s="78"/>
+      <c r="AK6" s="78"/>
+      <c r="AL6" s="78"/>
+      <c r="AM6" s="78"/>
+      <c r="AN6" s="78"/>
+      <c r="AO6" s="78"/>
+      <c r="AP6" s="78"/>
+      <c r="AQ6" s="78"/>
+      <c r="AR6" s="78"/>
+      <c r="AS6" s="78"/>
+      <c r="AT6" s="78"/>
+      <c r="AU6" s="78"/>
+      <c r="AV6" s="78"/>
+      <c r="AW6" s="78"/>
+      <c r="AX6" s="78"/>
+      <c r="AY6" s="78"/>
+      <c r="AZ6" s="78"/>
+      <c r="BA6" s="78"/>
+      <c r="BB6" s="78"/>
+      <c r="BC6" s="78"/>
+      <c r="BD6" s="78"/>
+      <c r="BE6" s="78"/>
+      <c r="BF6" s="78"/>
+      <c r="BG6" s="78"/>
+      <c r="BH6" s="78"/>
+      <c r="BI6" s="78"/>
+      <c r="BJ6" s="78"/>
+      <c r="BK6" s="78"/>
+      <c r="BL6" s="78"/>
+      <c r="BM6" s="78"/>
+      <c r="BN6" s="78"/>
+      <c r="BO6" s="78"/>
+      <c r="BP6" s="78"/>
+      <c r="BQ6" s="78"/>
+      <c r="BR6" s="78"/>
+      <c r="BS6" s="78"/>
+      <c r="BT6" s="78"/>
+      <c r="BU6" s="78"/>
+      <c r="BV6" s="78"/>
+      <c r="BW6" s="78"/>
+      <c r="BX6" s="78"/>
+      <c r="BY6" s="78"/>
+      <c r="BZ6" s="78"/>
+      <c r="CA6" s="78"/>
+      <c r="CB6" s="78"/>
+      <c r="CC6" s="78"/>
+      <c r="CD6" s="78"/>
+      <c r="CE6" s="78"/>
     </row>
     <row r="7" spans="1:84" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="72" t="s">
+      <c r="A7" s="61" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="18" t="s">
@@ -2251,132 +2338,132 @@
       <c r="C7" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="64" t="s">
+      <c r="D7" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="62">
+      <c r="E7" s="73"/>
+      <c r="F7" s="73"/>
+      <c r="G7" s="73"/>
+      <c r="H7" s="74">
         <v>45992</v>
       </c>
-      <c r="I7" s="62"/>
-      <c r="J7" s="62"/>
-      <c r="K7" s="63"/>
-      <c r="L7" s="64" t="s">
+      <c r="I7" s="74"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="75"/>
+      <c r="L7" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="M7" s="65"/>
-      <c r="N7" s="65"/>
-      <c r="O7" s="65"/>
-      <c r="P7" s="62">
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="73"/>
+      <c r="P7" s="74">
         <v>45993</v>
       </c>
-      <c r="Q7" s="62"/>
-      <c r="R7" s="62"/>
-      <c r="S7" s="63"/>
-      <c r="T7" s="64" t="s">
+      <c r="Q7" s="74"/>
+      <c r="R7" s="74"/>
+      <c r="S7" s="75"/>
+      <c r="T7" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="U7" s="65"/>
-      <c r="V7" s="65"/>
-      <c r="W7" s="65"/>
-      <c r="X7" s="62">
+      <c r="U7" s="73"/>
+      <c r="V7" s="73"/>
+      <c r="W7" s="73"/>
+      <c r="X7" s="74">
         <v>45999</v>
       </c>
-      <c r="Y7" s="62"/>
-      <c r="Z7" s="62"/>
-      <c r="AA7" s="63"/>
-      <c r="AB7" s="64" t="s">
+      <c r="Y7" s="74"/>
+      <c r="Z7" s="74"/>
+      <c r="AA7" s="75"/>
+      <c r="AB7" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="AC7" s="65"/>
-      <c r="AD7" s="65"/>
-      <c r="AE7" s="65"/>
-      <c r="AF7" s="62">
+      <c r="AC7" s="73"/>
+      <c r="AD7" s="73"/>
+      <c r="AE7" s="73"/>
+      <c r="AF7" s="74">
         <v>46000</v>
       </c>
-      <c r="AG7" s="62"/>
-      <c r="AH7" s="62"/>
-      <c r="AI7" s="63"/>
-      <c r="AJ7" s="64" t="s">
+      <c r="AG7" s="74"/>
+      <c r="AH7" s="74"/>
+      <c r="AI7" s="75"/>
+      <c r="AJ7" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="AK7" s="65"/>
-      <c r="AL7" s="65"/>
-      <c r="AM7" s="65"/>
-      <c r="AN7" s="62">
+      <c r="AK7" s="73"/>
+      <c r="AL7" s="73"/>
+      <c r="AM7" s="73"/>
+      <c r="AN7" s="74">
         <v>46006</v>
       </c>
-      <c r="AO7" s="62"/>
-      <c r="AP7" s="62"/>
-      <c r="AQ7" s="63"/>
-      <c r="AR7" s="64" t="s">
+      <c r="AO7" s="74"/>
+      <c r="AP7" s="74"/>
+      <c r="AQ7" s="75"/>
+      <c r="AR7" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="AS7" s="65"/>
-      <c r="AT7" s="65"/>
-      <c r="AU7" s="65"/>
-      <c r="AV7" s="62">
+      <c r="AS7" s="73"/>
+      <c r="AT7" s="73"/>
+      <c r="AU7" s="73"/>
+      <c r="AV7" s="74">
         <v>46007</v>
       </c>
-      <c r="AW7" s="62"/>
-      <c r="AX7" s="62"/>
-      <c r="AY7" s="63"/>
-      <c r="AZ7" s="64" t="s">
+      <c r="AW7" s="74"/>
+      <c r="AX7" s="74"/>
+      <c r="AY7" s="75"/>
+      <c r="AZ7" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="BA7" s="65"/>
-      <c r="BB7" s="65"/>
-      <c r="BC7" s="65"/>
-      <c r="BD7" s="62">
+      <c r="BA7" s="73"/>
+      <c r="BB7" s="73"/>
+      <c r="BC7" s="73"/>
+      <c r="BD7" s="74">
         <v>46027</v>
       </c>
-      <c r="BE7" s="62"/>
-      <c r="BF7" s="62"/>
-      <c r="BG7" s="63"/>
-      <c r="BH7" s="64" t="s">
+      <c r="BE7" s="74"/>
+      <c r="BF7" s="74"/>
+      <c r="BG7" s="75"/>
+      <c r="BH7" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="BI7" s="65"/>
-      <c r="BJ7" s="65"/>
-      <c r="BK7" s="65"/>
-      <c r="BL7" s="62">
+      <c r="BI7" s="73"/>
+      <c r="BJ7" s="73"/>
+      <c r="BK7" s="73"/>
+      <c r="BL7" s="74">
         <v>46028</v>
       </c>
-      <c r="BM7" s="62"/>
-      <c r="BN7" s="62"/>
-      <c r="BO7" s="63"/>
-      <c r="BP7" s="64" t="s">
+      <c r="BM7" s="74"/>
+      <c r="BN7" s="74"/>
+      <c r="BO7" s="75"/>
+      <c r="BP7" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="BQ7" s="65"/>
-      <c r="BR7" s="65"/>
-      <c r="BS7" s="65"/>
-      <c r="BT7" s="62">
+      <c r="BQ7" s="73"/>
+      <c r="BR7" s="73"/>
+      <c r="BS7" s="73"/>
+      <c r="BT7" s="74">
         <v>46034</v>
       </c>
-      <c r="BU7" s="62"/>
-      <c r="BV7" s="62"/>
-      <c r="BW7" s="63"/>
-      <c r="BX7" s="64" t="s">
+      <c r="BU7" s="74"/>
+      <c r="BV7" s="74"/>
+      <c r="BW7" s="75"/>
+      <c r="BX7" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="BY7" s="65"/>
-      <c r="BZ7" s="65"/>
-      <c r="CA7" s="65"/>
-      <c r="CB7" s="62">
+      <c r="BY7" s="73"/>
+      <c r="BZ7" s="73"/>
+      <c r="CA7" s="73"/>
+      <c r="CB7" s="74">
         <v>46035</v>
       </c>
-      <c r="CC7" s="62"/>
-      <c r="CD7" s="62"/>
-      <c r="CE7" s="63"/>
-      <c r="CF7" s="71" t="s">
+      <c r="CC7" s="74"/>
+      <c r="CD7" s="74"/>
+      <c r="CE7" s="75"/>
+      <c r="CF7" s="60" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:84" ht="13" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="73"/>
+      <c r="A8" s="62"/>
       <c r="B8" s="19" t="s">
         <v>11</v>
       </c>
@@ -2623,7 +2710,7 @@
       <c r="CE8" s="7">
         <v>8</v>
       </c>
-      <c r="CF8" s="71"/>
+      <c r="CF8" s="60"/>
     </row>
     <row r="9" spans="1:84" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="35" t="s">
@@ -2633,10 +2720,10 @@
         <v>29</v>
       </c>
       <c r="C9" s="8"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="83"/>
-      <c r="F9" s="83"/>
-      <c r="G9" s="83"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
+      <c r="G9" s="76"/>
       <c r="H9" s="44"/>
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
@@ -2649,16 +2736,16 @@
       <c r="Q9" s="44"/>
       <c r="R9" s="44"/>
       <c r="S9" s="44"/>
-      <c r="T9" s="74" t="s">
+      <c r="T9" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="U9" s="75"/>
-      <c r="V9" s="75"/>
-      <c r="W9" s="75"/>
-      <c r="X9" s="75"/>
-      <c r="Y9" s="75"/>
-      <c r="Z9" s="75"/>
-      <c r="AA9" s="76"/>
+      <c r="U9" s="64"/>
+      <c r="V9" s="64"/>
+      <c r="W9" s="64"/>
+      <c r="X9" s="64"/>
+      <c r="Y9" s="64"/>
+      <c r="Z9" s="64"/>
+      <c r="AA9" s="65"/>
       <c r="AB9" s="44"/>
       <c r="AC9" s="44"/>
       <c r="AD9" s="44"/>
@@ -2715,7 +2802,7 @@
       <c r="CC9" s="44"/>
       <c r="CD9" s="44"/>
       <c r="CE9" s="44"/>
-      <c r="CF9" s="71"/>
+      <c r="CF9" s="60"/>
     </row>
     <row r="10" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="36" t="s">
@@ -2729,10 +2816,10 @@
       <c r="E10" s="44"/>
       <c r="F10" s="44"/>
       <c r="G10" s="44"/>
-      <c r="H10" s="83"/>
-      <c r="I10" s="83"/>
-      <c r="J10" s="83"/>
-      <c r="K10" s="83"/>
+      <c r="H10" s="76"/>
+      <c r="I10" s="76"/>
+      <c r="J10" s="76"/>
+      <c r="K10" s="76"/>
       <c r="L10" s="44"/>
       <c r="M10" s="44"/>
       <c r="N10" s="44"/>
@@ -2741,14 +2828,14 @@
       <c r="Q10" s="44"/>
       <c r="R10" s="44"/>
       <c r="S10" s="44"/>
-      <c r="T10" s="77"/>
-      <c r="U10" s="78"/>
-      <c r="V10" s="78"/>
-      <c r="W10" s="78"/>
-      <c r="X10" s="78"/>
-      <c r="Y10" s="78"/>
-      <c r="Z10" s="78"/>
-      <c r="AA10" s="79"/>
+      <c r="T10" s="66"/>
+      <c r="U10" s="67"/>
+      <c r="V10" s="67"/>
+      <c r="W10" s="67"/>
+      <c r="X10" s="67"/>
+      <c r="Y10" s="67"/>
+      <c r="Z10" s="67"/>
+      <c r="AA10" s="68"/>
       <c r="AB10" s="44"/>
       <c r="AC10" s="44"/>
       <c r="AD10" s="44"/>
@@ -2805,7 +2892,7 @@
       <c r="CC10" s="44"/>
       <c r="CD10" s="44"/>
       <c r="CE10" s="44"/>
-      <c r="CF10" s="71"/>
+      <c r="CF10" s="60"/>
     </row>
     <row r="11" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="36" t="s">
@@ -2831,14 +2918,14 @@
       <c r="Q11" s="44"/>
       <c r="R11" s="44"/>
       <c r="S11" s="44"/>
-      <c r="T11" s="77"/>
-      <c r="U11" s="78"/>
-      <c r="V11" s="78"/>
-      <c r="W11" s="78"/>
-      <c r="X11" s="78"/>
-      <c r="Y11" s="78"/>
-      <c r="Z11" s="78"/>
-      <c r="AA11" s="79"/>
+      <c r="T11" s="66"/>
+      <c r="U11" s="67"/>
+      <c r="V11" s="67"/>
+      <c r="W11" s="67"/>
+      <c r="X11" s="67"/>
+      <c r="Y11" s="67"/>
+      <c r="Z11" s="67"/>
+      <c r="AA11" s="68"/>
       <c r="AB11" s="44"/>
       <c r="AC11" s="44"/>
       <c r="AD11" s="44"/>
@@ -2895,7 +2982,7 @@
       <c r="CC11" s="44"/>
       <c r="CD11" s="44"/>
       <c r="CE11" s="44"/>
-      <c r="CF11" s="71"/>
+      <c r="CF11" s="60"/>
     </row>
     <row r="12" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
@@ -2921,14 +3008,14 @@
       <c r="Q12" s="44"/>
       <c r="R12" s="44"/>
       <c r="S12" s="44"/>
-      <c r="T12" s="77"/>
-      <c r="U12" s="78"/>
-      <c r="V12" s="78"/>
-      <c r="W12" s="78"/>
-      <c r="X12" s="78"/>
-      <c r="Y12" s="78"/>
-      <c r="Z12" s="78"/>
-      <c r="AA12" s="79"/>
+      <c r="T12" s="66"/>
+      <c r="U12" s="67"/>
+      <c r="V12" s="67"/>
+      <c r="W12" s="67"/>
+      <c r="X12" s="67"/>
+      <c r="Y12" s="67"/>
+      <c r="Z12" s="67"/>
+      <c r="AA12" s="68"/>
       <c r="AB12" s="44"/>
       <c r="AC12" s="44"/>
       <c r="AD12" s="44"/>
@@ -2985,7 +3072,7 @@
       <c r="CC12" s="44"/>
       <c r="CD12" s="44"/>
       <c r="CE12" s="44"/>
-      <c r="CF12" s="71"/>
+      <c r="CF12" s="60"/>
     </row>
     <row r="13" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A13" s="58" t="s">
@@ -3011,14 +3098,14 @@
       <c r="Q13" s="44"/>
       <c r="R13" s="44"/>
       <c r="S13" s="44"/>
-      <c r="T13" s="77"/>
-      <c r="U13" s="78"/>
-      <c r="V13" s="78"/>
-      <c r="W13" s="78"/>
-      <c r="X13" s="78"/>
-      <c r="Y13" s="78"/>
-      <c r="Z13" s="78"/>
-      <c r="AA13" s="79"/>
+      <c r="T13" s="66"/>
+      <c r="U13" s="67"/>
+      <c r="V13" s="67"/>
+      <c r="W13" s="67"/>
+      <c r="X13" s="67"/>
+      <c r="Y13" s="67"/>
+      <c r="Z13" s="67"/>
+      <c r="AA13" s="68"/>
       <c r="AB13" s="44"/>
       <c r="AC13" s="44"/>
       <c r="AD13" s="44"/>
@@ -3075,7 +3162,7 @@
       <c r="CC13" s="44"/>
       <c r="CD13" s="44"/>
       <c r="CE13" s="44"/>
-      <c r="CF13" s="71"/>
+      <c r="CF13" s="60"/>
     </row>
     <row r="14" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A14" s="58" t="s">
@@ -3101,14 +3188,14 @@
       <c r="Q14" s="44"/>
       <c r="R14" s="44"/>
       <c r="S14" s="44"/>
-      <c r="T14" s="77"/>
-      <c r="U14" s="78"/>
-      <c r="V14" s="78"/>
-      <c r="W14" s="78"/>
-      <c r="X14" s="78"/>
-      <c r="Y14" s="78"/>
-      <c r="Z14" s="78"/>
-      <c r="AA14" s="79"/>
+      <c r="T14" s="66"/>
+      <c r="U14" s="67"/>
+      <c r="V14" s="67"/>
+      <c r="W14" s="67"/>
+      <c r="X14" s="67"/>
+      <c r="Y14" s="67"/>
+      <c r="Z14" s="67"/>
+      <c r="AA14" s="68"/>
       <c r="AB14" s="45" t="s">
         <v>39</v>
       </c>
@@ -3167,7 +3254,7 @@
       <c r="CC14" s="44"/>
       <c r="CD14" s="44"/>
       <c r="CE14" s="44"/>
-      <c r="CF14" s="71"/>
+      <c r="CF14" s="60"/>
     </row>
     <row r="15" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A15" s="58" t="s">
@@ -3193,14 +3280,14 @@
       <c r="Q15" s="44"/>
       <c r="R15" s="44"/>
       <c r="S15" s="44"/>
-      <c r="T15" s="77"/>
-      <c r="U15" s="78"/>
-      <c r="V15" s="78"/>
-      <c r="W15" s="78"/>
-      <c r="X15" s="78"/>
-      <c r="Y15" s="78"/>
-      <c r="Z15" s="78"/>
-      <c r="AA15" s="79"/>
+      <c r="T15" s="66"/>
+      <c r="U15" s="67"/>
+      <c r="V15" s="67"/>
+      <c r="W15" s="67"/>
+      <c r="X15" s="67"/>
+      <c r="Y15" s="67"/>
+      <c r="Z15" s="67"/>
+      <c r="AA15" s="68"/>
       <c r="AB15" s="44"/>
       <c r="AC15" s="45" t="s">
         <v>39</v>
@@ -3267,7 +3354,7 @@
       <c r="CC15" s="44"/>
       <c r="CD15" s="44"/>
       <c r="CE15" s="44"/>
-      <c r="CF15" s="71"/>
+      <c r="CF15" s="60"/>
     </row>
     <row r="16" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A16" s="30" t="s">
@@ -3291,14 +3378,14 @@
       <c r="Q16" s="44"/>
       <c r="R16" s="44"/>
       <c r="S16" s="44"/>
-      <c r="T16" s="77"/>
-      <c r="U16" s="78"/>
-      <c r="V16" s="78"/>
-      <c r="W16" s="78"/>
-      <c r="X16" s="78"/>
-      <c r="Y16" s="78"/>
-      <c r="Z16" s="78"/>
-      <c r="AA16" s="79"/>
+      <c r="T16" s="66"/>
+      <c r="U16" s="67"/>
+      <c r="V16" s="67"/>
+      <c r="W16" s="67"/>
+      <c r="X16" s="67"/>
+      <c r="Y16" s="67"/>
+      <c r="Z16" s="67"/>
+      <c r="AA16" s="68"/>
       <c r="AB16" s="44"/>
       <c r="AC16" s="44"/>
       <c r="AD16" s="44"/>
@@ -3355,7 +3442,7 @@
       <c r="CC16" s="44"/>
       <c r="CD16" s="44"/>
       <c r="CE16" s="44"/>
-      <c r="CF16" s="71"/>
+      <c r="CF16" s="60"/>
     </row>
     <row r="17" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A17" s="28" t="s">
@@ -3379,14 +3466,14 @@
       <c r="Q17" s="44"/>
       <c r="R17" s="44"/>
       <c r="S17" s="44"/>
-      <c r="T17" s="77"/>
-      <c r="U17" s="78"/>
-      <c r="V17" s="78"/>
-      <c r="W17" s="78"/>
-      <c r="X17" s="78"/>
-      <c r="Y17" s="78"/>
-      <c r="Z17" s="78"/>
-      <c r="AA17" s="79"/>
+      <c r="T17" s="66"/>
+      <c r="U17" s="67"/>
+      <c r="V17" s="67"/>
+      <c r="W17" s="67"/>
+      <c r="X17" s="67"/>
+      <c r="Y17" s="67"/>
+      <c r="Z17" s="67"/>
+      <c r="AA17" s="68"/>
       <c r="AB17" s="44"/>
       <c r="AC17" s="44"/>
       <c r="AD17" s="44"/>
@@ -3453,7 +3540,7 @@
       <c r="CC17" s="44"/>
       <c r="CD17" s="44"/>
       <c r="CE17" s="44"/>
-      <c r="CF17" s="71"/>
+      <c r="CF17" s="60"/>
     </row>
     <row r="18" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A18" s="28" t="s">
@@ -3477,14 +3564,14 @@
       <c r="Q18" s="44"/>
       <c r="R18" s="44"/>
       <c r="S18" s="44"/>
-      <c r="T18" s="77"/>
-      <c r="U18" s="78"/>
-      <c r="V18" s="78"/>
-      <c r="W18" s="78"/>
-      <c r="X18" s="78"/>
-      <c r="Y18" s="78"/>
-      <c r="Z18" s="78"/>
-      <c r="AA18" s="79"/>
+      <c r="T18" s="66"/>
+      <c r="U18" s="67"/>
+      <c r="V18" s="67"/>
+      <c r="W18" s="67"/>
+      <c r="X18" s="67"/>
+      <c r="Y18" s="67"/>
+      <c r="Z18" s="67"/>
+      <c r="AA18" s="68"/>
       <c r="AB18" s="44"/>
       <c r="AC18" s="44"/>
       <c r="AD18" s="44"/>
@@ -3547,7 +3634,7 @@
       <c r="CC18" s="44"/>
       <c r="CD18" s="44"/>
       <c r="CE18" s="44"/>
-      <c r="CF18" s="71"/>
+      <c r="CF18" s="60"/>
     </row>
     <row r="19" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A19" s="28" t="s">
@@ -3571,14 +3658,14 @@
       <c r="Q19" s="44"/>
       <c r="R19" s="44"/>
       <c r="S19" s="44"/>
-      <c r="T19" s="77"/>
-      <c r="U19" s="78"/>
-      <c r="V19" s="78"/>
-      <c r="W19" s="78"/>
-      <c r="X19" s="78"/>
-      <c r="Y19" s="78"/>
-      <c r="Z19" s="78"/>
-      <c r="AA19" s="79"/>
+      <c r="T19" s="66"/>
+      <c r="U19" s="67"/>
+      <c r="V19" s="67"/>
+      <c r="W19" s="67"/>
+      <c r="X19" s="67"/>
+      <c r="Y19" s="67"/>
+      <c r="Z19" s="67"/>
+      <c r="AA19" s="68"/>
       <c r="AB19" s="44"/>
       <c r="AC19" s="44"/>
       <c r="AD19" s="44"/>
@@ -3643,11 +3730,11 @@
       <c r="CC19" s="44"/>
       <c r="CD19" s="44"/>
       <c r="CE19" s="44"/>
-      <c r="CF19" s="71"/>
+      <c r="CF19" s="60"/>
     </row>
-    <row r="20" spans="1:84" ht="13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A20" s="28" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B20" s="16"/>
       <c r="C20" s="9"/>
@@ -3667,14 +3754,14 @@
       <c r="Q20" s="44"/>
       <c r="R20" s="44"/>
       <c r="S20" s="44"/>
-      <c r="T20" s="77"/>
-      <c r="U20" s="78"/>
-      <c r="V20" s="78"/>
-      <c r="W20" s="78"/>
-      <c r="X20" s="78"/>
-      <c r="Y20" s="78"/>
-      <c r="Z20" s="78"/>
-      <c r="AA20" s="79"/>
+      <c r="T20" s="66"/>
+      <c r="U20" s="67"/>
+      <c r="V20" s="67"/>
+      <c r="W20" s="67"/>
+      <c r="X20" s="67"/>
+      <c r="Y20" s="67"/>
+      <c r="Z20" s="67"/>
+      <c r="AA20" s="68"/>
       <c r="AB20" s="44"/>
       <c r="AC20" s="44"/>
       <c r="AD20" s="44"/>
@@ -3691,10 +3778,10 @@
       <c r="AO20" s="44"/>
       <c r="AP20" s="44"/>
       <c r="AQ20" s="44"/>
-      <c r="AR20" s="44"/>
-      <c r="AS20" s="44"/>
-      <c r="AT20" s="44"/>
-      <c r="AU20" s="44"/>
+      <c r="AR20" s="54"/>
+      <c r="AS20" s="54"/>
+      <c r="AT20" s="54"/>
+      <c r="AU20" s="54"/>
       <c r="AV20" s="44"/>
       <c r="AW20" s="44"/>
       <c r="AX20" s="44"/>
@@ -3703,30 +3790,14 @@
       <c r="BA20" s="44"/>
       <c r="BB20" s="44"/>
       <c r="BC20" s="44"/>
-      <c r="BD20" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="BE20" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="BF20" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="BG20" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="BH20" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="BI20" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="BJ20" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="BK20" s="46" t="s">
-        <v>41</v>
-      </c>
+      <c r="BD20" s="44"/>
+      <c r="BE20" s="44"/>
+      <c r="BF20" s="44"/>
+      <c r="BG20" s="44"/>
+      <c r="BH20" s="44"/>
+      <c r="BI20" s="44"/>
+      <c r="BJ20" s="44"/>
+      <c r="BK20" s="44"/>
       <c r="BL20" s="44"/>
       <c r="BM20" s="44"/>
       <c r="BN20" s="44"/>
@@ -3735,8 +3806,12 @@
       <c r="BQ20" s="44"/>
       <c r="BR20" s="44"/>
       <c r="BS20" s="44"/>
-      <c r="BT20" s="44"/>
-      <c r="BU20" s="44"/>
+      <c r="BT20" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="BU20" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="BV20" s="44"/>
       <c r="BW20" s="44"/>
       <c r="BX20" s="44"/>
@@ -3747,11 +3822,11 @@
       <c r="CC20" s="44"/>
       <c r="CD20" s="44"/>
       <c r="CE20" s="44"/>
-      <c r="CF20" s="71"/>
+      <c r="CF20" s="60"/>
     </row>
     <row r="21" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A21" s="37" t="s">
-        <v>35</v>
+      <c r="A21" s="28" t="s">
+        <v>59</v>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="9"/>
@@ -3771,14 +3846,14 @@
       <c r="Q21" s="44"/>
       <c r="R21" s="44"/>
       <c r="S21" s="44"/>
-      <c r="T21" s="77"/>
-      <c r="U21" s="78"/>
-      <c r="V21" s="78"/>
-      <c r="W21" s="78"/>
-      <c r="X21" s="78"/>
-      <c r="Y21" s="78"/>
-      <c r="Z21" s="78"/>
-      <c r="AA21" s="79"/>
+      <c r="T21" s="66"/>
+      <c r="U21" s="67"/>
+      <c r="V21" s="67"/>
+      <c r="W21" s="67"/>
+      <c r="X21" s="67"/>
+      <c r="Y21" s="67"/>
+      <c r="Z21" s="67"/>
+      <c r="AA21" s="68"/>
       <c r="AB21" s="44"/>
       <c r="AC21" s="44"/>
       <c r="AD21" s="44"/>
@@ -3807,18 +3882,46 @@
       <c r="BA21" s="44"/>
       <c r="BB21" s="44"/>
       <c r="BC21" s="44"/>
-      <c r="BD21" s="44"/>
-      <c r="BE21" s="44"/>
-      <c r="BF21" s="44"/>
-      <c r="BG21" s="44"/>
+      <c r="BD21" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="BE21" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="BF21" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="BG21" s="49" t="s">
+        <v>40</v>
+      </c>
+      <c r="BH21" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BI21" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BJ21" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BK21" s="46" t="s">
+        <v>41</v>
+      </c>
       <c r="BL21" s="44"/>
       <c r="BM21" s="44"/>
       <c r="BN21" s="44"/>
       <c r="BO21" s="44"/>
-      <c r="BP21" s="44"/>
-      <c r="BQ21" s="44"/>
-      <c r="BR21" s="44"/>
-      <c r="BS21" s="44"/>
+      <c r="BP21" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BQ21" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BR21" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BS21" s="46" t="s">
+        <v>41</v>
+      </c>
       <c r="BT21" s="44"/>
       <c r="BU21" s="44"/>
       <c r="BV21" s="44"/>
@@ -3831,11 +3934,11 @@
       <c r="CC21" s="44"/>
       <c r="CD21" s="44"/>
       <c r="CE21" s="44"/>
-      <c r="CF21" s="71"/>
+      <c r="CF21" s="60"/>
     </row>
     <row r="22" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A22" s="36" t="s">
-        <v>48</v>
+      <c r="A22" s="37" t="s">
+        <v>35</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="9"/>
@@ -3855,14 +3958,14 @@
       <c r="Q22" s="44"/>
       <c r="R22" s="44"/>
       <c r="S22" s="44"/>
-      <c r="T22" s="77"/>
-      <c r="U22" s="78"/>
-      <c r="V22" s="78"/>
-      <c r="W22" s="78"/>
-      <c r="X22" s="78"/>
-      <c r="Y22" s="78"/>
-      <c r="Z22" s="78"/>
-      <c r="AA22" s="79"/>
+      <c r="T22" s="66"/>
+      <c r="U22" s="67"/>
+      <c r="V22" s="67"/>
+      <c r="W22" s="67"/>
+      <c r="X22" s="67"/>
+      <c r="Y22" s="67"/>
+      <c r="Z22" s="67"/>
+      <c r="AA22" s="68"/>
       <c r="AB22" s="44"/>
       <c r="AC22" s="44"/>
       <c r="AD22" s="44"/>
@@ -3871,15 +3974,11 @@
       <c r="AG22" s="44"/>
       <c r="AH22" s="44"/>
       <c r="AI22" s="44"/>
-      <c r="AJ22" s="46"/>
-      <c r="AK22" s="46"/>
-      <c r="AL22" s="46"/>
-      <c r="AM22" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="AN22" s="44" t="s">
-        <v>41</v>
-      </c>
+      <c r="AJ22" s="44"/>
+      <c r="AK22" s="44"/>
+      <c r="AL22" s="44"/>
+      <c r="AM22" s="44"/>
+      <c r="AN22" s="44"/>
       <c r="AO22" s="44"/>
       <c r="AP22" s="44"/>
       <c r="AQ22" s="44"/>
@@ -3899,10 +3998,6 @@
       <c r="BE22" s="44"/>
       <c r="BF22" s="44"/>
       <c r="BG22" s="44"/>
-      <c r="BH22" s="44"/>
-      <c r="BI22" s="44"/>
-      <c r="BJ22" s="44"/>
-      <c r="BK22" s="44"/>
       <c r="BL22" s="44"/>
       <c r="BM22" s="44"/>
       <c r="BN22" s="44"/>
@@ -3923,11 +4018,11 @@
       <c r="CC22" s="44"/>
       <c r="CD22" s="44"/>
       <c r="CE22" s="44"/>
-      <c r="CF22" s="71"/>
+      <c r="CF22" s="60"/>
     </row>
     <row r="23" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A23" s="43" t="s">
-        <v>49</v>
+      <c r="A23" s="36" t="s">
+        <v>48</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="9"/>
@@ -3947,14 +4042,14 @@
       <c r="Q23" s="44"/>
       <c r="R23" s="44"/>
       <c r="S23" s="44"/>
-      <c r="T23" s="77"/>
-      <c r="U23" s="78"/>
-      <c r="V23" s="78"/>
-      <c r="W23" s="78"/>
-      <c r="X23" s="78"/>
-      <c r="Y23" s="78"/>
-      <c r="Z23" s="78"/>
-      <c r="AA23" s="79"/>
+      <c r="T23" s="66"/>
+      <c r="U23" s="67"/>
+      <c r="V23" s="67"/>
+      <c r="W23" s="67"/>
+      <c r="X23" s="67"/>
+      <c r="Y23" s="67"/>
+      <c r="Z23" s="67"/>
+      <c r="AA23" s="68"/>
       <c r="AB23" s="44"/>
       <c r="AC23" s="44"/>
       <c r="AD23" s="44"/>
@@ -3963,11 +4058,15 @@
       <c r="AG23" s="44"/>
       <c r="AH23" s="44"/>
       <c r="AI23" s="44"/>
-      <c r="AJ23" s="44"/>
-      <c r="AK23" s="44"/>
-      <c r="AL23" s="44"/>
-      <c r="AM23" s="44"/>
-      <c r="AN23" s="44"/>
+      <c r="AJ23" s="46"/>
+      <c r="AK23" s="46"/>
+      <c r="AL23" s="46"/>
+      <c r="AM23" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="AN23" s="44" t="s">
+        <v>41</v>
+      </c>
       <c r="AO23" s="44"/>
       <c r="AP23" s="44"/>
       <c r="AQ23" s="44"/>
@@ -3987,6 +4086,7 @@
       <c r="BE23" s="44"/>
       <c r="BF23" s="44"/>
       <c r="BG23" s="44"/>
+      <c r="BH23" s="44"/>
       <c r="BI23" s="44"/>
       <c r="BJ23" s="44"/>
       <c r="BK23" s="44"/>
@@ -4010,11 +4110,11 @@
       <c r="CC23" s="44"/>
       <c r="CD23" s="44"/>
       <c r="CE23" s="44"/>
-      <c r="CF23" s="71"/>
+      <c r="CF23" s="60"/>
     </row>
     <row r="24" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A24" s="38" t="s">
-        <v>50</v>
+      <c r="A24" s="43" t="s">
+        <v>49</v>
       </c>
       <c r="B24" s="16"/>
       <c r="C24" s="9"/>
@@ -4034,14 +4134,14 @@
       <c r="Q24" s="44"/>
       <c r="R24" s="44"/>
       <c r="S24" s="44"/>
-      <c r="T24" s="77"/>
-      <c r="U24" s="78"/>
-      <c r="V24" s="78"/>
-      <c r="W24" s="78"/>
-      <c r="X24" s="78"/>
-      <c r="Y24" s="78"/>
-      <c r="Z24" s="78"/>
-      <c r="AA24" s="79"/>
+      <c r="T24" s="66"/>
+      <c r="U24" s="67"/>
+      <c r="V24" s="67"/>
+      <c r="W24" s="67"/>
+      <c r="X24" s="67"/>
+      <c r="Y24" s="67"/>
+      <c r="Z24" s="67"/>
+      <c r="AA24" s="68"/>
       <c r="AB24" s="44"/>
       <c r="AC24" s="44"/>
       <c r="AD24" s="44"/>
@@ -4074,7 +4174,6 @@
       <c r="BE24" s="44"/>
       <c r="BF24" s="44"/>
       <c r="BG24" s="44"/>
-      <c r="BH24" s="44"/>
       <c r="BI24" s="44"/>
       <c r="BJ24" s="44"/>
       <c r="BK24" s="44"/>
@@ -4098,11 +4197,11 @@
       <c r="CC24" s="44"/>
       <c r="CD24" s="44"/>
       <c r="CE24" s="44"/>
-      <c r="CF24" s="71"/>
+      <c r="CF24" s="60"/>
     </row>
     <row r="25" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A25" s="36" t="s">
-        <v>51</v>
+      <c r="A25" s="38" t="s">
+        <v>50</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="9"/>
@@ -4122,14 +4221,14 @@
       <c r="Q25" s="44"/>
       <c r="R25" s="44"/>
       <c r="S25" s="44"/>
-      <c r="T25" s="77"/>
-      <c r="U25" s="78"/>
-      <c r="V25" s="78"/>
-      <c r="W25" s="78"/>
-      <c r="X25" s="78"/>
-      <c r="Y25" s="78"/>
-      <c r="Z25" s="78"/>
-      <c r="AA25" s="79"/>
+      <c r="T25" s="66"/>
+      <c r="U25" s="67"/>
+      <c r="V25" s="67"/>
+      <c r="W25" s="67"/>
+      <c r="X25" s="67"/>
+      <c r="Y25" s="67"/>
+      <c r="Z25" s="67"/>
+      <c r="AA25" s="68"/>
       <c r="AB25" s="44"/>
       <c r="AC25" s="44"/>
       <c r="AD25" s="44"/>
@@ -4149,13 +4248,11 @@
       <c r="AR25" s="44"/>
       <c r="AS25" s="44"/>
       <c r="AT25" s="44"/>
-      <c r="AU25" s="46" t="s">
-        <v>41</v>
-      </c>
+      <c r="AU25" s="44"/>
       <c r="AV25" s="44"/>
       <c r="AW25" s="44"/>
       <c r="AX25" s="44"/>
-      <c r="AY25" s="34"/>
+      <c r="AY25" s="44"/>
       <c r="AZ25" s="44"/>
       <c r="BA25" s="44"/>
       <c r="BB25" s="44"/>
@@ -4188,11 +4285,11 @@
       <c r="CC25" s="44"/>
       <c r="CD25" s="44"/>
       <c r="CE25" s="44"/>
-      <c r="CF25" s="71"/>
+      <c r="CF25" s="60"/>
     </row>
     <row r="26" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A26" s="38" t="s">
-        <v>52</v>
+      <c r="A26" s="36" t="s">
+        <v>51</v>
       </c>
       <c r="B26" s="16"/>
       <c r="C26" s="9"/>
@@ -4212,14 +4309,14 @@
       <c r="Q26" s="44"/>
       <c r="R26" s="44"/>
       <c r="S26" s="44"/>
-      <c r="T26" s="77"/>
-      <c r="U26" s="78"/>
-      <c r="V26" s="78"/>
-      <c r="W26" s="78"/>
-      <c r="X26" s="78"/>
-      <c r="Y26" s="78"/>
-      <c r="Z26" s="78"/>
-      <c r="AA26" s="79"/>
+      <c r="T26" s="66"/>
+      <c r="U26" s="67"/>
+      <c r="V26" s="67"/>
+      <c r="W26" s="67"/>
+      <c r="X26" s="67"/>
+      <c r="Y26" s="67"/>
+      <c r="Z26" s="67"/>
+      <c r="AA26" s="68"/>
       <c r="AB26" s="44"/>
       <c r="AC26" s="44"/>
       <c r="AD26" s="44"/>
@@ -4239,11 +4336,13 @@
       <c r="AR26" s="44"/>
       <c r="AS26" s="44"/>
       <c r="AT26" s="44"/>
-      <c r="AU26" s="44"/>
+      <c r="AU26" s="46" t="s">
+        <v>41</v>
+      </c>
       <c r="AV26" s="44"/>
       <c r="AW26" s="44"/>
       <c r="AX26" s="44"/>
-      <c r="AY26" s="44"/>
+      <c r="AY26" s="34"/>
       <c r="AZ26" s="44"/>
       <c r="BA26" s="44"/>
       <c r="BB26" s="44"/>
@@ -4260,14 +4359,14 @@
       <c r="BM26" s="44"/>
       <c r="BN26" s="44"/>
       <c r="BO26" s="44"/>
-      <c r="BP26" s="57"/>
-      <c r="BQ26" s="57"/>
-      <c r="BR26" s="57"/>
-      <c r="BS26" s="57"/>
-      <c r="BT26" s="57"/>
-      <c r="BU26" s="57"/>
-      <c r="BV26" s="57"/>
-      <c r="BW26" s="57"/>
+      <c r="BP26" s="44"/>
+      <c r="BQ26" s="44"/>
+      <c r="BR26" s="44"/>
+      <c r="BS26" s="44"/>
+      <c r="BT26" s="44"/>
+      <c r="BU26" s="44"/>
+      <c r="BV26" s="44"/>
+      <c r="BW26" s="44"/>
       <c r="BX26" s="44"/>
       <c r="BY26" s="44"/>
       <c r="BZ26" s="44"/>
@@ -4276,11 +4375,11 @@
       <c r="CC26" s="44"/>
       <c r="CD26" s="44"/>
       <c r="CE26" s="44"/>
-      <c r="CF26" s="71"/>
+      <c r="CF26" s="60"/>
     </row>
     <row r="27" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A27" s="30" t="s">
-        <v>36</v>
+      <c r="A27" s="38" t="s">
+        <v>52</v>
       </c>
       <c r="B27" s="16"/>
       <c r="C27" s="9"/>
@@ -4300,14 +4399,14 @@
       <c r="Q27" s="44"/>
       <c r="R27" s="44"/>
       <c r="S27" s="44"/>
-      <c r="T27" s="77"/>
-      <c r="U27" s="78"/>
-      <c r="V27" s="78"/>
-      <c r="W27" s="78"/>
-      <c r="X27" s="78"/>
-      <c r="Y27" s="78"/>
-      <c r="Z27" s="78"/>
-      <c r="AA27" s="79"/>
+      <c r="T27" s="66"/>
+      <c r="U27" s="67"/>
+      <c r="V27" s="67"/>
+      <c r="W27" s="67"/>
+      <c r="X27" s="67"/>
+      <c r="Y27" s="67"/>
+      <c r="Z27" s="67"/>
+      <c r="AA27" s="68"/>
       <c r="AB27" s="44"/>
       <c r="AC27" s="44"/>
       <c r="AD27" s="44"/>
@@ -4348,14 +4447,14 @@
       <c r="BM27" s="44"/>
       <c r="BN27" s="44"/>
       <c r="BO27" s="44"/>
-      <c r="BP27" s="44"/>
-      <c r="BQ27" s="44"/>
-      <c r="BR27" s="44"/>
-      <c r="BS27" s="44"/>
-      <c r="BT27" s="44"/>
-      <c r="BU27" s="44"/>
-      <c r="BV27" s="44"/>
-      <c r="BW27" s="44"/>
+      <c r="BP27" s="57"/>
+      <c r="BQ27" s="57"/>
+      <c r="BR27" s="57"/>
+      <c r="BS27" s="57"/>
+      <c r="BT27" s="57"/>
+      <c r="BU27" s="57"/>
+      <c r="BV27" s="57"/>
+      <c r="BW27" s="57"/>
       <c r="BX27" s="44"/>
       <c r="BY27" s="44"/>
       <c r="BZ27" s="44"/>
@@ -4364,11 +4463,11 @@
       <c r="CC27" s="44"/>
       <c r="CD27" s="44"/>
       <c r="CE27" s="44"/>
-      <c r="CF27" s="71"/>
+      <c r="CF27" s="60"/>
     </row>
     <row r="28" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A28" s="28" t="s">
-        <v>56</v>
+      <c r="A28" s="30" t="s">
+        <v>36</v>
       </c>
       <c r="B28" s="16"/>
       <c r="C28" s="9"/>
@@ -4388,14 +4487,14 @@
       <c r="Q28" s="44"/>
       <c r="R28" s="44"/>
       <c r="S28" s="44"/>
-      <c r="T28" s="77"/>
-      <c r="U28" s="78"/>
-      <c r="V28" s="78"/>
-      <c r="W28" s="78"/>
-      <c r="X28" s="78"/>
-      <c r="Y28" s="78"/>
-      <c r="Z28" s="78"/>
-      <c r="AA28" s="79"/>
+      <c r="T28" s="66"/>
+      <c r="U28" s="67"/>
+      <c r="V28" s="67"/>
+      <c r="W28" s="67"/>
+      <c r="X28" s="67"/>
+      <c r="Y28" s="67"/>
+      <c r="Z28" s="67"/>
+      <c r="AA28" s="68"/>
       <c r="AB28" s="44"/>
       <c r="AC28" s="44"/>
       <c r="AD28" s="44"/>
@@ -4408,25 +4507,13 @@
       <c r="AK28" s="44"/>
       <c r="AL28" s="44"/>
       <c r="AM28" s="44"/>
-      <c r="AN28" s="46"/>
-      <c r="AO28" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="AP28" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="AQ28" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="AR28" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="AS28" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="AT28" s="46" t="s">
-        <v>41</v>
-      </c>
+      <c r="AN28" s="44"/>
+      <c r="AO28" s="44"/>
+      <c r="AP28" s="44"/>
+      <c r="AQ28" s="44"/>
+      <c r="AR28" s="44"/>
+      <c r="AS28" s="44"/>
+      <c r="AT28" s="44"/>
       <c r="AU28" s="44"/>
       <c r="AV28" s="44"/>
       <c r="AW28" s="44"/>
@@ -4464,11 +4551,11 @@
       <c r="CC28" s="44"/>
       <c r="CD28" s="44"/>
       <c r="CE28" s="44"/>
-      <c r="CF28" s="71"/>
+      <c r="CF28" s="60"/>
     </row>
     <row r="29" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A29" s="28" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="9"/>
@@ -4488,14 +4575,14 @@
       <c r="Q29" s="44"/>
       <c r="R29" s="44"/>
       <c r="S29" s="44"/>
-      <c r="T29" s="77"/>
-      <c r="U29" s="78"/>
-      <c r="V29" s="78"/>
-      <c r="W29" s="78"/>
-      <c r="X29" s="78"/>
-      <c r="Y29" s="78"/>
-      <c r="Z29" s="78"/>
-      <c r="AA29" s="79"/>
+      <c r="T29" s="66"/>
+      <c r="U29" s="67"/>
+      <c r="V29" s="67"/>
+      <c r="W29" s="67"/>
+      <c r="X29" s="67"/>
+      <c r="Y29" s="67"/>
+      <c r="Z29" s="67"/>
+      <c r="AA29" s="68"/>
       <c r="AB29" s="44"/>
       <c r="AC29" s="44"/>
       <c r="AD29" s="44"/>
@@ -4508,41 +4595,33 @@
       <c r="AK29" s="44"/>
       <c r="AL29" s="44"/>
       <c r="AM29" s="44"/>
-      <c r="AN29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="AO29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="AP29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="AQ29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="AR29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="AS29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="AT29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="AU29" s="45" t="s">
-        <v>57</v>
-      </c>
+      <c r="AN29" s="46"/>
+      <c r="AO29" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP29" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ29" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="AR29" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="AS29" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="AT29" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="AU29" s="44"/>
       <c r="AV29" s="44"/>
       <c r="AW29" s="44"/>
       <c r="AX29" s="44"/>
       <c r="AY29" s="44"/>
       <c r="AZ29" s="44"/>
-      <c r="BA29" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="BB29" s="45" t="s">
-        <v>57</v>
-      </c>
+      <c r="BA29" s="44"/>
+      <c r="BB29" s="44"/>
       <c r="BC29" s="44"/>
       <c r="BD29" s="44"/>
       <c r="BE29" s="44"/>
@@ -4572,11 +4651,11 @@
       <c r="CC29" s="44"/>
       <c r="CD29" s="44"/>
       <c r="CE29" s="44"/>
-      <c r="CF29" s="71"/>
+      <c r="CF29" s="60"/>
     </row>
     <row r="30" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A30" s="42" t="s">
-        <v>58</v>
+      <c r="A30" s="28" t="s">
+        <v>60</v>
       </c>
       <c r="B30" s="16"/>
       <c r="C30" s="9"/>
@@ -4596,14 +4675,14 @@
       <c r="Q30" s="44"/>
       <c r="R30" s="44"/>
       <c r="S30" s="44"/>
-      <c r="T30" s="77"/>
-      <c r="U30" s="78"/>
-      <c r="V30" s="78"/>
-      <c r="W30" s="78"/>
-      <c r="X30" s="78"/>
-      <c r="Y30" s="78"/>
-      <c r="Z30" s="78"/>
-      <c r="AA30" s="79"/>
+      <c r="T30" s="66"/>
+      <c r="U30" s="67"/>
+      <c r="V30" s="67"/>
+      <c r="W30" s="67"/>
+      <c r="X30" s="67"/>
+      <c r="Y30" s="67"/>
+      <c r="Z30" s="67"/>
+      <c r="AA30" s="68"/>
       <c r="AB30" s="44"/>
       <c r="AC30" s="44"/>
       <c r="AD30" s="44"/>
@@ -4616,48 +4695,50 @@
       <c r="AK30" s="44"/>
       <c r="AL30" s="44"/>
       <c r="AM30" s="44"/>
-      <c r="AN30" s="44"/>
-      <c r="AO30" s="44"/>
-      <c r="AP30" s="44"/>
-      <c r="AQ30" s="44"/>
-      <c r="AR30" s="44"/>
-      <c r="AS30" s="44"/>
-      <c r="AT30" s="44"/>
-      <c r="AU30" s="44"/>
+      <c r="AN30" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="AO30" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="AP30" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="AQ30" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="AR30" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="AS30" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="AT30" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="AU30" s="45" t="s">
+        <v>57</v>
+      </c>
       <c r="AV30" s="44"/>
       <c r="AW30" s="44"/>
       <c r="AX30" s="44"/>
       <c r="AY30" s="44"/>
       <c r="AZ30" s="44"/>
-      <c r="BA30" s="44"/>
-      <c r="BB30" s="44"/>
-      <c r="BC30" s="45" t="s">
+      <c r="BA30" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="BD30" s="45" t="s">
+      <c r="BB30" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="BE30" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="BF30" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="BG30" s="45" t="s">
-        <v>57</v>
-      </c>
-      <c r="BH30" s="44" t="s">
-        <v>57</v>
-      </c>
-      <c r="BI30" s="44" t="s">
-        <v>57</v>
-      </c>
-      <c r="BJ30" s="44" t="s">
-        <v>57</v>
-      </c>
-      <c r="BK30" s="44" t="s">
-        <v>57</v>
-      </c>
+      <c r="BC30" s="44"/>
+      <c r="BD30" s="44"/>
+      <c r="BE30" s="44"/>
+      <c r="BF30" s="44"/>
+      <c r="BG30" s="44"/>
+      <c r="BH30" s="44"/>
+      <c r="BI30" s="44"/>
+      <c r="BJ30" s="44"/>
+      <c r="BK30" s="44"/>
       <c r="BL30" s="44"/>
       <c r="BM30" s="44"/>
       <c r="BN30" s="44"/>
@@ -4678,11 +4759,11 @@
       <c r="CC30" s="44"/>
       <c r="CD30" s="44"/>
       <c r="CE30" s="44"/>
-      <c r="CF30" s="71"/>
+      <c r="CF30" s="60"/>
     </row>
     <row r="31" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A31" s="42" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B31" s="16"/>
       <c r="C31" s="9"/>
@@ -4702,14 +4783,14 @@
       <c r="Q31" s="44"/>
       <c r="R31" s="44"/>
       <c r="S31" s="44"/>
-      <c r="T31" s="77"/>
-      <c r="U31" s="78"/>
-      <c r="V31" s="78"/>
-      <c r="W31" s="78"/>
-      <c r="X31" s="78"/>
-      <c r="Y31" s="78"/>
-      <c r="Z31" s="78"/>
-      <c r="AA31" s="79"/>
+      <c r="T31" s="66"/>
+      <c r="U31" s="67"/>
+      <c r="V31" s="67"/>
+      <c r="W31" s="67"/>
+      <c r="X31" s="67"/>
+      <c r="Y31" s="67"/>
+      <c r="Z31" s="67"/>
+      <c r="AA31" s="68"/>
       <c r="AB31" s="44"/>
       <c r="AC31" s="44"/>
       <c r="AD31" s="44"/>
@@ -4737,21 +4818,33 @@
       <c r="AZ31" s="44"/>
       <c r="BA31" s="44"/>
       <c r="BB31" s="44"/>
-      <c r="BC31" s="44"/>
-      <c r="BD31" s="44"/>
-      <c r="BE31" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="BF31" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="BG31" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="BH31" s="44"/>
-      <c r="BI31" s="44"/>
-      <c r="BJ31" s="44"/>
-      <c r="BK31" s="44"/>
+      <c r="BC31" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="BD31" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="BE31" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="BF31" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG31" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="BH31" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="BI31" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="BJ31" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="BK31" s="44" t="s">
+        <v>57</v>
+      </c>
       <c r="BL31" s="44"/>
       <c r="BM31" s="44"/>
       <c r="BN31" s="44"/>
@@ -4772,11 +4865,11 @@
       <c r="CC31" s="44"/>
       <c r="CD31" s="44"/>
       <c r="CE31" s="44"/>
-      <c r="CF31" s="71"/>
+      <c r="CF31" s="60"/>
     </row>
     <row r="32" spans="1:84" ht="13" x14ac:dyDescent="0.3">
       <c r="A32" s="42" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B32" s="16"/>
       <c r="C32" s="9"/>
@@ -4796,14 +4889,14 @@
       <c r="Q32" s="44"/>
       <c r="R32" s="44"/>
       <c r="S32" s="44"/>
-      <c r="T32" s="77"/>
-      <c r="U32" s="78"/>
-      <c r="V32" s="78"/>
-      <c r="W32" s="78"/>
-      <c r="X32" s="78"/>
-      <c r="Y32" s="78"/>
-      <c r="Z32" s="78"/>
-      <c r="AA32" s="79"/>
+      <c r="T32" s="66"/>
+      <c r="U32" s="67"/>
+      <c r="V32" s="67"/>
+      <c r="W32" s="67"/>
+      <c r="X32" s="67"/>
+      <c r="Y32" s="67"/>
+      <c r="Z32" s="67"/>
+      <c r="AA32" s="68"/>
       <c r="AB32" s="44"/>
       <c r="AC32" s="44"/>
       <c r="AD32" s="44"/>
@@ -4829,21 +4922,19 @@
       <c r="AX32" s="44"/>
       <c r="AY32" s="44"/>
       <c r="AZ32" s="44"/>
-      <c r="BA32" s="46" t="s">
+      <c r="BA32" s="44"/>
+      <c r="BB32" s="44"/>
+      <c r="BC32" s="44"/>
+      <c r="BD32" s="44"/>
+      <c r="BE32" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="BB32" s="46" t="s">
+      <c r="BF32" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="BC32" s="46" t="s">
+      <c r="BG32" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="BD32" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="BE32" s="3"/>
-      <c r="BF32" s="44"/>
-      <c r="BG32" s="44"/>
       <c r="BH32" s="44"/>
       <c r="BI32" s="44"/>
       <c r="BJ32" s="44"/>
@@ -4868,11 +4959,11 @@
       <c r="CC32" s="44"/>
       <c r="CD32" s="44"/>
       <c r="CE32" s="44"/>
-      <c r="CF32" s="71"/>
+      <c r="CF32" s="60"/>
     </row>
     <row r="33" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A33" s="28" t="s">
-        <v>55</v>
+      <c r="A33" s="42" t="s">
+        <v>53</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="9"/>
@@ -4892,14 +4983,14 @@
       <c r="Q33" s="44"/>
       <c r="R33" s="44"/>
       <c r="S33" s="44"/>
-      <c r="T33" s="77"/>
-      <c r="U33" s="78"/>
-      <c r="V33" s="78"/>
-      <c r="W33" s="78"/>
-      <c r="X33" s="78"/>
-      <c r="Y33" s="78"/>
-      <c r="Z33" s="78"/>
-      <c r="AA33" s="79"/>
+      <c r="T33" s="66"/>
+      <c r="U33" s="67"/>
+      <c r="V33" s="67"/>
+      <c r="W33" s="67"/>
+      <c r="X33" s="67"/>
+      <c r="Y33" s="67"/>
+      <c r="Z33" s="67"/>
+      <c r="AA33" s="68"/>
       <c r="AB33" s="44"/>
       <c r="AC33" s="44"/>
       <c r="AD33" s="44"/>
@@ -4925,11 +5016,19 @@
       <c r="AX33" s="44"/>
       <c r="AY33" s="44"/>
       <c r="AZ33" s="44"/>
-      <c r="BA33" s="44"/>
-      <c r="BB33" s="44"/>
-      <c r="BC33" s="44"/>
-      <c r="BD33" s="44"/>
-      <c r="BE33" s="44"/>
+      <c r="BA33" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BB33" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BC33" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BD33" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="BE33" s="3"/>
       <c r="BF33" s="44"/>
       <c r="BG33" s="44"/>
       <c r="BH33" s="44"/>
@@ -4956,15 +5055,13 @@
       <c r="CC33" s="44"/>
       <c r="CD33" s="44"/>
       <c r="CE33" s="44"/>
-      <c r="CF33" s="71"/>
+      <c r="CF33" s="60"/>
     </row>
     <row r="34" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A34" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="B34" s="16" t="s">
-        <v>30</v>
-      </c>
+      <c r="A34" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="16"/>
       <c r="C34" s="9"/>
       <c r="D34" s="44"/>
       <c r="E34" s="44"/>
@@ -4982,14 +5079,14 @@
       <c r="Q34" s="44"/>
       <c r="R34" s="44"/>
       <c r="S34" s="44"/>
-      <c r="T34" s="77"/>
-      <c r="U34" s="78"/>
-      <c r="V34" s="78"/>
-      <c r="W34" s="78"/>
-      <c r="X34" s="78"/>
-      <c r="Y34" s="78"/>
-      <c r="Z34" s="78"/>
-      <c r="AA34" s="79"/>
+      <c r="T34" s="66"/>
+      <c r="U34" s="67"/>
+      <c r="V34" s="67"/>
+      <c r="W34" s="67"/>
+      <c r="X34" s="67"/>
+      <c r="Y34" s="67"/>
+      <c r="Z34" s="67"/>
+      <c r="AA34" s="68"/>
       <c r="AB34" s="44"/>
       <c r="AC34" s="44"/>
       <c r="AD34" s="44"/>
@@ -5046,14 +5143,14 @@
       <c r="CC34" s="44"/>
       <c r="CD34" s="44"/>
       <c r="CE34" s="44"/>
-      <c r="CF34" s="71"/>
+      <c r="CF34" s="60"/>
     </row>
-    <row r="35" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A35" s="32" t="s">
-        <v>22</v>
+    <row r="35" spans="1:84" ht="13" x14ac:dyDescent="0.3">
+      <c r="A35" s="31" t="s">
+        <v>21</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="44"/>
@@ -5064,30 +5161,22 @@
       <c r="I35" s="44"/>
       <c r="J35" s="44"/>
       <c r="K35" s="44"/>
-      <c r="L35" s="49" t="s">
-        <v>39</v>
-      </c>
-      <c r="M35" s="49" t="s">
-        <v>39</v>
-      </c>
-      <c r="N35" s="49" t="s">
-        <v>39</v>
-      </c>
-      <c r="O35" s="49" t="s">
-        <v>39</v>
-      </c>
+      <c r="L35" s="44"/>
+      <c r="M35" s="44"/>
+      <c r="N35" s="44"/>
+      <c r="O35" s="44"/>
       <c r="P35" s="44"/>
       <c r="Q35" s="44"/>
       <c r="R35" s="44"/>
       <c r="S35" s="44"/>
-      <c r="T35" s="77"/>
-      <c r="U35" s="78"/>
-      <c r="V35" s="78"/>
-      <c r="W35" s="78"/>
-      <c r="X35" s="78"/>
-      <c r="Y35" s="78"/>
-      <c r="Z35" s="78"/>
-      <c r="AA35" s="79"/>
+      <c r="T35" s="66"/>
+      <c r="U35" s="67"/>
+      <c r="V35" s="67"/>
+      <c r="W35" s="67"/>
+      <c r="X35" s="67"/>
+      <c r="Y35" s="67"/>
+      <c r="Z35" s="67"/>
+      <c r="AA35" s="68"/>
       <c r="AB35" s="44"/>
       <c r="AC35" s="44"/>
       <c r="AD35" s="44"/>
@@ -5144,11 +5233,11 @@
       <c r="CC35" s="44"/>
       <c r="CD35" s="44"/>
       <c r="CE35" s="44"/>
-      <c r="CF35" s="71"/>
+      <c r="CF35" s="60"/>
     </row>
     <row r="36" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A36" s="32" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B36" s="16" t="s">
         <v>29</v>
@@ -5162,30 +5251,30 @@
       <c r="I36" s="44"/>
       <c r="J36" s="44"/>
       <c r="K36" s="44"/>
-      <c r="L36" s="45" t="s">
+      <c r="L36" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="M36" s="45" t="s">
+      <c r="M36" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="N36" s="45" t="s">
+      <c r="N36" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="O36" s="45" t="s">
+      <c r="O36" s="49" t="s">
         <v>39</v>
       </c>
       <c r="P36" s="44"/>
       <c r="Q36" s="44"/>
       <c r="R36" s="44"/>
       <c r="S36" s="44"/>
-      <c r="T36" s="77"/>
-      <c r="U36" s="78"/>
-      <c r="V36" s="78"/>
-      <c r="W36" s="78"/>
-      <c r="X36" s="78"/>
-      <c r="Y36" s="78"/>
-      <c r="Z36" s="78"/>
-      <c r="AA36" s="79"/>
+      <c r="T36" s="66"/>
+      <c r="U36" s="67"/>
+      <c r="V36" s="67"/>
+      <c r="W36" s="67"/>
+      <c r="X36" s="67"/>
+      <c r="Y36" s="67"/>
+      <c r="Z36" s="67"/>
+      <c r="AA36" s="68"/>
       <c r="AB36" s="44"/>
       <c r="AC36" s="44"/>
       <c r="AD36" s="44"/>
@@ -5242,11 +5331,11 @@
       <c r="CC36" s="44"/>
       <c r="CD36" s="44"/>
       <c r="CE36" s="44"/>
-      <c r="CF36" s="71"/>
+      <c r="CF36" s="60"/>
     </row>
     <row r="37" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A37" s="32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B37" s="16" t="s">
         <v>29</v>
@@ -5260,36 +5349,32 @@
       <c r="I37" s="44"/>
       <c r="J37" s="44"/>
       <c r="K37" s="44"/>
-      <c r="L37" s="46" t="s">
+      <c r="L37" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="M37" s="46" t="s">
+      <c r="M37" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="N37" s="46" t="s">
+      <c r="N37" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="O37" s="46" t="s">
+      <c r="O37" s="45" t="s">
         <v>39</v>
       </c>
       <c r="P37" s="44"/>
       <c r="Q37" s="44"/>
       <c r="R37" s="44"/>
       <c r="S37" s="44"/>
-      <c r="T37" s="77"/>
-      <c r="U37" s="78"/>
-      <c r="V37" s="78"/>
-      <c r="W37" s="78"/>
-      <c r="X37" s="78"/>
-      <c r="Y37" s="78"/>
-      <c r="Z37" s="78"/>
-      <c r="AA37" s="79"/>
-      <c r="AB37" s="46" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC37" s="46" t="s">
-        <v>39</v>
-      </c>
+      <c r="T37" s="66"/>
+      <c r="U37" s="67"/>
+      <c r="V37" s="67"/>
+      <c r="W37" s="67"/>
+      <c r="X37" s="67"/>
+      <c r="Y37" s="67"/>
+      <c r="Z37" s="67"/>
+      <c r="AA37" s="68"/>
+      <c r="AB37" s="44"/>
+      <c r="AC37" s="44"/>
       <c r="AD37" s="44"/>
       <c r="AE37" s="44"/>
       <c r="AF37" s="44"/>
@@ -5308,7 +5393,7 @@
       <c r="AS37" s="44"/>
       <c r="AT37" s="44"/>
       <c r="AU37" s="44"/>
-      <c r="AV37" s="3"/>
+      <c r="AV37" s="44"/>
       <c r="AW37" s="44"/>
       <c r="AX37" s="44"/>
       <c r="AY37" s="44"/>
@@ -5344,14 +5429,14 @@
       <c r="CC37" s="44"/>
       <c r="CD37" s="44"/>
       <c r="CE37" s="44"/>
-      <c r="CF37" s="71"/>
+      <c r="CF37" s="60"/>
     </row>
     <row r="38" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A38" s="32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="44"/>
@@ -5362,24 +5447,36 @@
       <c r="I38" s="44"/>
       <c r="J38" s="44"/>
       <c r="K38" s="44"/>
-      <c r="L38" s="44"/>
-      <c r="M38" s="44"/>
-      <c r="N38" s="44"/>
-      <c r="O38" s="44"/>
+      <c r="L38" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="M38" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="N38" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="O38" s="46" t="s">
+        <v>39</v>
+      </c>
       <c r="P38" s="44"/>
       <c r="Q38" s="44"/>
       <c r="R38" s="44"/>
       <c r="S38" s="44"/>
-      <c r="T38" s="77"/>
-      <c r="U38" s="78"/>
-      <c r="V38" s="78"/>
-      <c r="W38" s="78"/>
-      <c r="X38" s="78"/>
-      <c r="Y38" s="78"/>
-      <c r="Z38" s="78"/>
-      <c r="AA38" s="79"/>
-      <c r="AB38" s="47"/>
-      <c r="AC38" s="44"/>
+      <c r="T38" s="66"/>
+      <c r="U38" s="67"/>
+      <c r="V38" s="67"/>
+      <c r="W38" s="67"/>
+      <c r="X38" s="67"/>
+      <c r="Y38" s="67"/>
+      <c r="Z38" s="67"/>
+      <c r="AA38" s="68"/>
+      <c r="AB38" s="46" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC38" s="46" t="s">
+        <v>39</v>
+      </c>
       <c r="AD38" s="44"/>
       <c r="AE38" s="44"/>
       <c r="AF38" s="44"/>
@@ -5394,10 +5491,10 @@
       <c r="AO38" s="44"/>
       <c r="AP38" s="44"/>
       <c r="AQ38" s="44"/>
-      <c r="AR38" s="49"/>
-      <c r="AS38" s="49"/>
-      <c r="AT38" s="49"/>
-      <c r="AU38" s="49"/>
+      <c r="AR38" s="44"/>
+      <c r="AS38" s="44"/>
+      <c r="AT38" s="44"/>
+      <c r="AU38" s="44"/>
       <c r="AV38" s="3"/>
       <c r="AW38" s="44"/>
       <c r="AX38" s="44"/>
@@ -5434,11 +5531,11 @@
       <c r="CC38" s="44"/>
       <c r="CD38" s="44"/>
       <c r="CE38" s="44"/>
-      <c r="CF38" s="71"/>
+      <c r="CF38" s="60"/>
     </row>
     <row r="39" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A39" s="32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B39" s="16" t="s">
         <v>30</v>
@@ -5460,22 +5557,18 @@
       <c r="Q39" s="44"/>
       <c r="R39" s="44"/>
       <c r="S39" s="44"/>
-      <c r="T39" s="77"/>
-      <c r="U39" s="78"/>
-      <c r="V39" s="78"/>
-      <c r="W39" s="78"/>
-      <c r="X39" s="78"/>
-      <c r="Y39" s="78"/>
-      <c r="Z39" s="78"/>
-      <c r="AA39" s="79"/>
-      <c r="AB39" s="44"/>
+      <c r="T39" s="66"/>
+      <c r="U39" s="67"/>
+      <c r="V39" s="67"/>
+      <c r="W39" s="67"/>
+      <c r="X39" s="67"/>
+      <c r="Y39" s="67"/>
+      <c r="Z39" s="67"/>
+      <c r="AA39" s="68"/>
+      <c r="AB39" s="47"/>
       <c r="AC39" s="44"/>
-      <c r="AD39" s="46" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE39" s="46" t="s">
-        <v>39</v>
-      </c>
+      <c r="AD39" s="44"/>
+      <c r="AE39" s="44"/>
       <c r="AF39" s="44"/>
       <c r="AG39" s="44"/>
       <c r="AH39" s="44"/>
@@ -5488,26 +5581,18 @@
       <c r="AO39" s="44"/>
       <c r="AP39" s="44"/>
       <c r="AQ39" s="44"/>
-      <c r="AR39" s="44"/>
-      <c r="AS39" s="44"/>
-      <c r="AT39" s="44"/>
-      <c r="AU39" s="44"/>
-      <c r="AV39" s="44"/>
+      <c r="AR39" s="49"/>
+      <c r="AS39" s="49"/>
+      <c r="AT39" s="49"/>
+      <c r="AU39" s="49"/>
+      <c r="AV39" s="3"/>
       <c r="AW39" s="44"/>
       <c r="AX39" s="44"/>
       <c r="AY39" s="44"/>
-      <c r="AZ39" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="BA39" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="BB39" s="49" t="s">
-        <v>40</v>
-      </c>
-      <c r="BC39" s="49" t="s">
-        <v>40</v>
-      </c>
+      <c r="AZ39" s="44"/>
+      <c r="BA39" s="44"/>
+      <c r="BB39" s="44"/>
+      <c r="BC39" s="44"/>
       <c r="BD39" s="44"/>
       <c r="BE39" s="44"/>
       <c r="BF39" s="44"/>
@@ -5536,128 +5621,100 @@
       <c r="CC39" s="44"/>
       <c r="CD39" s="44"/>
       <c r="CE39" s="44"/>
-      <c r="CF39" s="71"/>
+      <c r="CF39" s="60"/>
     </row>
     <row r="40" spans="1:84" x14ac:dyDescent="0.25">
       <c r="A40" s="32" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" s="16" t="s">
         <v>30</v>
       </c>
       <c r="C40" s="9"/>
-      <c r="D40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="E40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="F40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="G40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="H40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="I40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="J40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="K40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="L40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="M40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="N40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="O40" s="50" t="s">
-        <v>39</v>
-      </c>
+      <c r="D40" s="44"/>
+      <c r="E40" s="44"/>
+      <c r="F40" s="44"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="44"/>
+      <c r="I40" s="44"/>
+      <c r="J40" s="44"/>
+      <c r="K40" s="44"/>
+      <c r="L40" s="44"/>
+      <c r="M40" s="44"/>
+      <c r="N40" s="44"/>
+      <c r="O40" s="44"/>
       <c r="P40" s="44"/>
       <c r="Q40" s="44"/>
       <c r="R40" s="44"/>
       <c r="S40" s="44"/>
-      <c r="T40" s="77"/>
-      <c r="U40" s="78"/>
-      <c r="V40" s="78"/>
-      <c r="W40" s="78"/>
-      <c r="X40" s="78"/>
-      <c r="Y40" s="78"/>
-      <c r="Z40" s="78"/>
-      <c r="AA40" s="79"/>
-      <c r="AB40" s="50" t="s">
+      <c r="T40" s="66"/>
+      <c r="U40" s="67"/>
+      <c r="V40" s="67"/>
+      <c r="W40" s="67"/>
+      <c r="X40" s="67"/>
+      <c r="Y40" s="67"/>
+      <c r="Z40" s="67"/>
+      <c r="AA40" s="68"/>
+      <c r="AB40" s="44"/>
+      <c r="AC40" s="44"/>
+      <c r="AD40" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="AC40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD40" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="AE40" s="50" t="s">
+      <c r="AE40" s="46" t="s">
         <v>39</v>
       </c>
       <c r="AF40" s="44"/>
       <c r="AG40" s="44"/>
       <c r="AH40" s="44"/>
       <c r="AI40" s="44"/>
-      <c r="AJ40" s="53"/>
-      <c r="AK40" s="50"/>
-      <c r="AL40" s="50"/>
-      <c r="AM40" s="50"/>
-      <c r="AN40" s="50"/>
-      <c r="AO40" s="50"/>
-      <c r="AP40" s="50"/>
-      <c r="AQ40" s="50"/>
-      <c r="AR40" s="50"/>
-      <c r="AS40" s="50"/>
-      <c r="AT40" s="50"/>
-      <c r="AU40" s="50"/>
+      <c r="AJ40" s="44"/>
+      <c r="AK40" s="44"/>
+      <c r="AL40" s="44"/>
+      <c r="AM40" s="44"/>
+      <c r="AN40" s="44"/>
+      <c r="AO40" s="44"/>
+      <c r="AP40" s="44"/>
+      <c r="AQ40" s="44"/>
+      <c r="AR40" s="44"/>
+      <c r="AS40" s="44"/>
+      <c r="AT40" s="44"/>
+      <c r="AU40" s="44"/>
       <c r="AV40" s="44"/>
       <c r="AW40" s="44"/>
       <c r="AX40" s="44"/>
       <c r="AY40" s="44"/>
-      <c r="AZ40" s="50"/>
-      <c r="BA40" s="50"/>
-      <c r="BB40" s="50"/>
-      <c r="BC40" s="50"/>
-      <c r="BD40" s="50"/>
-      <c r="BE40" s="50"/>
-      <c r="BF40" s="50"/>
-      <c r="BG40" s="50"/>
-      <c r="BH40" s="50" t="s">
+      <c r="AZ40" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="BI40" s="50" t="s">
+      <c r="BA40" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="BJ40" s="50" t="s">
+      <c r="BB40" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="BK40" s="50" t="s">
+      <c r="BC40" s="49" t="s">
         <v>40</v>
       </c>
+      <c r="BD40" s="44"/>
+      <c r="BE40" s="44"/>
+      <c r="BF40" s="44"/>
+      <c r="BG40" s="44"/>
+      <c r="BH40" s="44"/>
+      <c r="BI40" s="44"/>
+      <c r="BJ40" s="44"/>
+      <c r="BK40" s="44"/>
       <c r="BL40" s="44"/>
       <c r="BM40" s="44"/>
       <c r="BN40" s="44"/>
       <c r="BO40" s="44"/>
-      <c r="BP40" s="50"/>
-      <c r="BQ40" s="50"/>
-      <c r="BR40" s="50"/>
-      <c r="BS40" s="50"/>
-      <c r="BT40" s="50"/>
-      <c r="BU40" s="50"/>
-      <c r="BV40" s="50"/>
-      <c r="BW40" s="50"/>
+      <c r="BP40" s="44"/>
+      <c r="BQ40" s="44"/>
+      <c r="BR40" s="44"/>
+      <c r="BS40" s="44"/>
+      <c r="BT40" s="44"/>
+      <c r="BU40" s="44"/>
+      <c r="BV40" s="44"/>
+      <c r="BW40" s="44"/>
       <c r="BX40" s="44"/>
       <c r="BY40" s="44"/>
       <c r="BZ40" s="44"/>
@@ -5666,90 +5723,128 @@
       <c r="CC40" s="44"/>
       <c r="CD40" s="44"/>
       <c r="CE40" s="44"/>
-      <c r="CF40" s="71"/>
+      <c r="CF40" s="60"/>
     </row>
     <row r="41" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A41" s="33" t="s">
-        <v>28</v>
+      <c r="A41" s="32" t="s">
+        <v>27</v>
       </c>
       <c r="B41" s="16" t="s">
         <v>30</v>
       </c>
       <c r="C41" s="9"/>
-      <c r="D41" s="44"/>
-      <c r="E41" s="44"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="44"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="44"/>
-      <c r="J41" s="44"/>
-      <c r="K41" s="44"/>
-      <c r="L41" s="44"/>
-      <c r="M41" s="44"/>
-      <c r="N41" s="44"/>
-      <c r="O41" s="44"/>
+      <c r="D41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="E41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="F41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="G41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="H41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="I41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="J41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="K41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="L41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="M41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="N41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="O41" s="50" t="s">
+        <v>39</v>
+      </c>
       <c r="P41" s="44"/>
       <c r="Q41" s="44"/>
       <c r="R41" s="44"/>
       <c r="S41" s="44"/>
-      <c r="T41" s="77"/>
-      <c r="U41" s="78"/>
-      <c r="V41" s="78"/>
-      <c r="W41" s="78"/>
-      <c r="X41" s="78"/>
-      <c r="Y41" s="78"/>
-      <c r="Z41" s="78"/>
-      <c r="AA41" s="79"/>
-      <c r="AB41" s="44"/>
-      <c r="AC41" s="3"/>
-      <c r="AD41" s="34"/>
-      <c r="AE41" s="45" t="s">
+      <c r="T41" s="66"/>
+      <c r="U41" s="67"/>
+      <c r="V41" s="67"/>
+      <c r="W41" s="67"/>
+      <c r="X41" s="67"/>
+      <c r="Y41" s="67"/>
+      <c r="Z41" s="67"/>
+      <c r="AA41" s="68"/>
+      <c r="AB41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD41" s="50" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE41" s="50" t="s">
         <v>39</v>
       </c>
       <c r="AF41" s="44"/>
       <c r="AG41" s="44"/>
       <c r="AH41" s="44"/>
       <c r="AI41" s="44"/>
-      <c r="AJ41" s="39"/>
-      <c r="AK41" s="45"/>
-      <c r="AL41" s="45"/>
-      <c r="AM41" s="45"/>
-      <c r="AN41" s="44"/>
-      <c r="AO41" s="44"/>
-      <c r="AP41" s="44"/>
-      <c r="AQ41" s="44"/>
-      <c r="AR41" s="44"/>
-      <c r="AS41" s="44"/>
-      <c r="AT41" s="44"/>
-      <c r="AU41" s="44"/>
+      <c r="AJ41" s="53"/>
+      <c r="AK41" s="50"/>
+      <c r="AL41" s="50"/>
+      <c r="AM41" s="50"/>
+      <c r="AN41" s="50"/>
+      <c r="AO41" s="50"/>
+      <c r="AP41" s="50"/>
+      <c r="AQ41" s="50"/>
+      <c r="AR41" s="50"/>
+      <c r="AS41" s="50"/>
+      <c r="AT41" s="50"/>
+      <c r="AU41" s="50"/>
       <c r="AV41" s="44"/>
       <c r="AW41" s="44"/>
       <c r="AX41" s="44"/>
       <c r="AY41" s="44"/>
-      <c r="AZ41" s="44"/>
-      <c r="BA41" s="44"/>
-      <c r="BB41" s="44"/>
-      <c r="BC41" s="44"/>
-      <c r="BD41" s="44"/>
-      <c r="BE41" s="44"/>
-      <c r="BF41" s="44"/>
-      <c r="BG41" s="44"/>
-      <c r="BH41" s="44"/>
-      <c r="BI41" s="44"/>
-      <c r="BJ41" s="44"/>
-      <c r="BK41" s="44"/>
+      <c r="AZ41" s="50"/>
+      <c r="BA41" s="50"/>
+      <c r="BB41" s="50"/>
+      <c r="BC41" s="50"/>
+      <c r="BD41" s="50"/>
+      <c r="BE41" s="50"/>
+      <c r="BF41" s="50"/>
+      <c r="BG41" s="50"/>
+      <c r="BH41" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="BI41" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="BJ41" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="BK41" s="50" t="s">
+        <v>40</v>
+      </c>
       <c r="BL41" s="44"/>
       <c r="BM41" s="44"/>
       <c r="BN41" s="44"/>
       <c r="BO41" s="44"/>
-      <c r="BP41" s="44"/>
-      <c r="BQ41" s="44"/>
-      <c r="BR41" s="44"/>
-      <c r="BS41" s="44"/>
-      <c r="BT41" s="44"/>
-      <c r="BU41" s="44"/>
-      <c r="BV41" s="44"/>
-      <c r="BW41" s="44"/>
+      <c r="BP41" s="50"/>
+      <c r="BQ41" s="50"/>
+      <c r="BR41" s="50"/>
+      <c r="BS41" s="50"/>
+      <c r="BT41" s="50"/>
+      <c r="BU41" s="50"/>
+      <c r="BV41" s="50"/>
+      <c r="BW41" s="50"/>
       <c r="BX41" s="44"/>
       <c r="BY41" s="44"/>
       <c r="BZ41" s="44"/>
@@ -5758,13 +5853,15 @@
       <c r="CC41" s="44"/>
       <c r="CD41" s="44"/>
       <c r="CE41" s="44"/>
-      <c r="CF41" s="71"/>
+      <c r="CF41" s="60"/>
     </row>
-    <row r="42" spans="1:84" ht="13" x14ac:dyDescent="0.3">
-      <c r="A42" s="40" t="s">
-        <v>32</v>
-      </c>
-      <c r="B42" s="16"/>
+    <row r="42" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A42" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="B42" s="16" t="s">
+        <v>30</v>
+      </c>
       <c r="C42" s="9"/>
       <c r="D42" s="44"/>
       <c r="E42" s="44"/>
@@ -5782,26 +5879,28 @@
       <c r="Q42" s="44"/>
       <c r="R42" s="44"/>
       <c r="S42" s="44"/>
-      <c r="T42" s="77"/>
-      <c r="U42" s="78"/>
-      <c r="V42" s="78"/>
-      <c r="W42" s="78"/>
-      <c r="X42" s="78"/>
-      <c r="Y42" s="78"/>
-      <c r="Z42" s="78"/>
-      <c r="AA42" s="79"/>
+      <c r="T42" s="66"/>
+      <c r="U42" s="67"/>
+      <c r="V42" s="67"/>
+      <c r="W42" s="67"/>
+      <c r="X42" s="67"/>
+      <c r="Y42" s="67"/>
+      <c r="Z42" s="67"/>
+      <c r="AA42" s="68"/>
       <c r="AB42" s="44"/>
-      <c r="AC42" s="44"/>
-      <c r="AD42" s="44"/>
-      <c r="AE42" s="48"/>
+      <c r="AC42" s="3"/>
+      <c r="AD42" s="34"/>
+      <c r="AE42" s="45" t="s">
+        <v>39</v>
+      </c>
       <c r="AF42" s="44"/>
       <c r="AG42" s="44"/>
       <c r="AH42" s="44"/>
       <c r="AI42" s="44"/>
-      <c r="AJ42" s="44"/>
-      <c r="AK42" s="44"/>
-      <c r="AL42" s="44"/>
-      <c r="AM42" s="44"/>
+      <c r="AJ42" s="39"/>
+      <c r="AK42" s="45"/>
+      <c r="AL42" s="45"/>
+      <c r="AM42" s="45"/>
       <c r="AN42" s="44"/>
       <c r="AO42" s="44"/>
       <c r="AP42" s="44"/>
@@ -5846,11 +5945,11 @@
       <c r="CC42" s="44"/>
       <c r="CD42" s="44"/>
       <c r="CE42" s="44"/>
-      <c r="CF42" s="71"/>
+      <c r="CF42" s="60"/>
     </row>
-    <row r="43" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A43" s="41" t="s">
-        <v>33</v>
+    <row r="43" spans="1:84" ht="13" x14ac:dyDescent="0.3">
+      <c r="A43" s="40" t="s">
+        <v>32</v>
       </c>
       <c r="B43" s="16"/>
       <c r="C43" s="9"/>
@@ -5870,18 +5969,18 @@
       <c r="Q43" s="44"/>
       <c r="R43" s="44"/>
       <c r="S43" s="44"/>
-      <c r="T43" s="77"/>
-      <c r="U43" s="78"/>
-      <c r="V43" s="78"/>
-      <c r="W43" s="78"/>
-      <c r="X43" s="78"/>
-      <c r="Y43" s="78"/>
-      <c r="Z43" s="78"/>
-      <c r="AA43" s="79"/>
+      <c r="T43" s="66"/>
+      <c r="U43" s="67"/>
+      <c r="V43" s="67"/>
+      <c r="W43" s="67"/>
+      <c r="X43" s="67"/>
+      <c r="Y43" s="67"/>
+      <c r="Z43" s="67"/>
+      <c r="AA43" s="68"/>
       <c r="AB43" s="44"/>
       <c r="AC43" s="44"/>
       <c r="AD43" s="44"/>
-      <c r="AE43" s="44"/>
+      <c r="AE43" s="48"/>
       <c r="AF43" s="44"/>
       <c r="AG43" s="44"/>
       <c r="AH43" s="44"/>
@@ -5926,20 +6025,22 @@
       <c r="BU43" s="44"/>
       <c r="BV43" s="44"/>
       <c r="BW43" s="44"/>
-      <c r="BX43" s="50"/>
-      <c r="BY43" s="50"/>
-      <c r="BZ43" s="50"/>
-      <c r="CA43" s="50"/>
+      <c r="BX43" s="44"/>
+      <c r="BY43" s="44"/>
+      <c r="BZ43" s="44"/>
+      <c r="CA43" s="44"/>
       <c r="CB43" s="44"/>
       <c r="CC43" s="44"/>
       <c r="CD43" s="44"/>
       <c r="CE43" s="44"/>
-      <c r="CF43" s="71"/>
+      <c r="CF43" s="60"/>
     </row>
-    <row r="44" spans="1:84" ht="13" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="10"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="11"/>
+    <row r="44" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A44" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="B44" s="16"/>
+      <c r="C44" s="9"/>
       <c r="D44" s="44"/>
       <c r="E44" s="44"/>
       <c r="F44" s="44"/>
@@ -5956,173 +6057,347 @@
       <c r="Q44" s="44"/>
       <c r="R44" s="44"/>
       <c r="S44" s="44"/>
-      <c r="T44" s="80"/>
-      <c r="U44" s="81"/>
-      <c r="V44" s="81"/>
-      <c r="W44" s="81"/>
-      <c r="X44" s="81"/>
-      <c r="Y44" s="81"/>
-      <c r="Z44" s="81"/>
-      <c r="AA44" s="82"/>
-      <c r="AB44" s="12"/>
-      <c r="AC44" s="13"/>
-      <c r="AD44" s="13"/>
-      <c r="AE44" s="13"/>
-      <c r="AF44" s="13"/>
-      <c r="AG44" s="13"/>
-      <c r="AH44" s="13"/>
-      <c r="AI44" s="14"/>
-      <c r="AJ44" s="12"/>
-      <c r="AK44" s="13"/>
-      <c r="AL44" s="13"/>
-      <c r="AM44" s="13"/>
-      <c r="AN44" s="13"/>
-      <c r="AO44" s="13"/>
-      <c r="AP44" s="13"/>
-      <c r="AQ44" s="14"/>
-      <c r="AR44" s="12"/>
-      <c r="AS44" s="13"/>
-      <c r="AT44" s="13"/>
-      <c r="AU44" s="13"/>
-      <c r="AV44" s="13"/>
-      <c r="AW44" s="13"/>
-      <c r="AX44" s="13"/>
-      <c r="AY44" s="14"/>
-      <c r="AZ44" s="12"/>
-      <c r="BA44" s="13"/>
-      <c r="BB44" s="13"/>
-      <c r="BC44" s="13"/>
-      <c r="BD44" s="13"/>
-      <c r="BE44" s="13"/>
-      <c r="BF44" s="13"/>
-      <c r="BG44" s="14"/>
-      <c r="BH44" s="12"/>
-      <c r="BI44" s="13"/>
-      <c r="BJ44" s="13"/>
-      <c r="BK44" s="13"/>
-      <c r="BL44" s="13"/>
-      <c r="BM44" s="13"/>
-      <c r="BN44" s="13"/>
-      <c r="BO44" s="14"/>
-      <c r="BP44" s="12"/>
-      <c r="BQ44" s="13"/>
-      <c r="BR44" s="13"/>
-      <c r="BS44" s="13"/>
-      <c r="BT44" s="13"/>
-      <c r="BU44" s="13"/>
-      <c r="BV44" s="13"/>
-      <c r="BW44" s="14"/>
-      <c r="BX44" s="12"/>
-      <c r="BY44" s="13"/>
-      <c r="BZ44" s="13"/>
-      <c r="CA44" s="13"/>
-      <c r="CB44" s="13"/>
-      <c r="CC44" s="13"/>
-      <c r="CD44" s="13"/>
-      <c r="CE44" s="14"/>
-      <c r="CF44" s="71"/>
+      <c r="T44" s="66"/>
+      <c r="U44" s="67"/>
+      <c r="V44" s="67"/>
+      <c r="W44" s="67"/>
+      <c r="X44" s="67"/>
+      <c r="Y44" s="67"/>
+      <c r="Z44" s="67"/>
+      <c r="AA44" s="68"/>
+      <c r="AB44" s="44"/>
+      <c r="AC44" s="44"/>
+      <c r="AD44" s="44"/>
+      <c r="AE44" s="44"/>
+      <c r="AF44" s="44"/>
+      <c r="AG44" s="44"/>
+      <c r="AH44" s="44"/>
+      <c r="AI44" s="44"/>
+      <c r="AJ44" s="44"/>
+      <c r="AK44" s="44"/>
+      <c r="AL44" s="44"/>
+      <c r="AM44" s="44"/>
+      <c r="AN44" s="44"/>
+      <c r="AO44" s="44"/>
+      <c r="AP44" s="44"/>
+      <c r="AQ44" s="44"/>
+      <c r="AR44" s="44"/>
+      <c r="AS44" s="44"/>
+      <c r="AT44" s="44"/>
+      <c r="AU44" s="44"/>
+      <c r="AV44" s="44"/>
+      <c r="AW44" s="44"/>
+      <c r="AX44" s="44"/>
+      <c r="AY44" s="44"/>
+      <c r="AZ44" s="44"/>
+      <c r="BA44" s="44"/>
+      <c r="BB44" s="44"/>
+      <c r="BC44" s="44"/>
+      <c r="BD44" s="44"/>
+      <c r="BE44" s="44"/>
+      <c r="BF44" s="44"/>
+      <c r="BG44" s="44"/>
+      <c r="BH44" s="44"/>
+      <c r="BI44" s="44"/>
+      <c r="BJ44" s="44"/>
+      <c r="BK44" s="44"/>
+      <c r="BL44" s="44"/>
+      <c r="BM44" s="44"/>
+      <c r="BN44" s="44"/>
+      <c r="BO44" s="44"/>
+      <c r="BP44" s="44"/>
+      <c r="BQ44" s="44"/>
+      <c r="BR44" s="44"/>
+      <c r="BS44" s="44"/>
+      <c r="BT44" s="44"/>
+      <c r="BU44" s="44"/>
+      <c r="BV44" s="44"/>
+      <c r="BW44" s="44"/>
+      <c r="BX44" s="50"/>
+      <c r="BY44" s="50"/>
+      <c r="BZ44" s="50"/>
+      <c r="CA44" s="50"/>
+      <c r="CB44" s="44"/>
+      <c r="CC44" s="44"/>
+      <c r="CD44" s="44"/>
+      <c r="CE44" s="44"/>
+      <c r="CF44" s="60"/>
     </row>
     <row r="45" spans="1:84" x14ac:dyDescent="0.25">
-      <c r="A45" s="70" t="s">
+      <c r="A45" s="84" t="s">
+        <v>63</v>
+      </c>
+      <c r="B45" s="85"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="44"/>
+      <c r="F45" s="44"/>
+      <c r="G45" s="44"/>
+      <c r="H45" s="44"/>
+      <c r="I45" s="44"/>
+      <c r="J45" s="44"/>
+      <c r="K45" s="44"/>
+      <c r="L45" s="44"/>
+      <c r="M45" s="44"/>
+      <c r="N45" s="44"/>
+      <c r="O45" s="44"/>
+      <c r="P45" s="44"/>
+      <c r="Q45" s="44"/>
+      <c r="R45" s="44"/>
+      <c r="S45" s="44"/>
+      <c r="T45" s="66"/>
+      <c r="U45" s="67"/>
+      <c r="V45" s="67"/>
+      <c r="W45" s="67"/>
+      <c r="X45" s="67"/>
+      <c r="Y45" s="67"/>
+      <c r="Z45" s="67"/>
+      <c r="AA45" s="68"/>
+      <c r="AB45" s="86"/>
+      <c r="AC45" s="87"/>
+      <c r="AD45" s="87"/>
+      <c r="AE45" s="87"/>
+      <c r="AF45" s="87"/>
+      <c r="AG45" s="87"/>
+      <c r="AH45" s="87"/>
+      <c r="AI45" s="88"/>
+      <c r="AJ45" s="86"/>
+      <c r="AK45" s="87"/>
+      <c r="AL45" s="87"/>
+      <c r="AM45" s="87"/>
+      <c r="AN45" s="87"/>
+      <c r="AO45" s="87"/>
+      <c r="AP45" s="87"/>
+      <c r="AQ45" s="88"/>
+      <c r="AR45" s="86"/>
+      <c r="AS45" s="87"/>
+      <c r="AT45" s="87"/>
+      <c r="AU45" s="87"/>
+      <c r="AV45" s="87"/>
+      <c r="AW45" s="87"/>
+      <c r="AX45" s="87"/>
+      <c r="AY45" s="88"/>
+      <c r="AZ45" s="86"/>
+      <c r="BA45" s="87"/>
+      <c r="BB45" s="87"/>
+      <c r="BC45" s="87"/>
+      <c r="BD45" s="87"/>
+      <c r="BE45" s="87"/>
+      <c r="BF45" s="87"/>
+      <c r="BG45" s="88"/>
+      <c r="BH45" s="86"/>
+      <c r="BI45" s="87"/>
+      <c r="BJ45" s="87"/>
+      <c r="BK45" s="87"/>
+      <c r="BL45" s="87"/>
+      <c r="BM45" s="87"/>
+      <c r="BN45" s="87"/>
+      <c r="BO45" s="88"/>
+      <c r="BP45" s="86"/>
+      <c r="BQ45" s="87"/>
+      <c r="BR45" s="87"/>
+      <c r="BS45" s="87"/>
+      <c r="BT45" s="87"/>
+      <c r="BU45" s="87"/>
+      <c r="BV45" s="91" t="s">
+        <v>41</v>
+      </c>
+      <c r="BW45" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="BX45" s="89"/>
+      <c r="BY45" s="90"/>
+      <c r="BZ45" s="90"/>
+      <c r="CA45" s="90"/>
+      <c r="CB45" s="87"/>
+      <c r="CC45" s="87"/>
+      <c r="CD45" s="87"/>
+      <c r="CE45" s="88"/>
+      <c r="CF45" s="60"/>
+    </row>
+    <row r="46" spans="1:84" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="10"/>
+      <c r="B46" s="17"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="44"/>
+      <c r="E46" s="44"/>
+      <c r="F46" s="44"/>
+      <c r="G46" s="44"/>
+      <c r="H46" s="44"/>
+      <c r="I46" s="44"/>
+      <c r="J46" s="44"/>
+      <c r="K46" s="44"/>
+      <c r="L46" s="44"/>
+      <c r="M46" s="44"/>
+      <c r="N46" s="44"/>
+      <c r="O46" s="44"/>
+      <c r="P46" s="44"/>
+      <c r="Q46" s="44"/>
+      <c r="R46" s="44"/>
+      <c r="S46" s="44"/>
+      <c r="T46" s="69"/>
+      <c r="U46" s="70"/>
+      <c r="V46" s="70"/>
+      <c r="W46" s="70"/>
+      <c r="X46" s="70"/>
+      <c r="Y46" s="70"/>
+      <c r="Z46" s="70"/>
+      <c r="AA46" s="71"/>
+      <c r="AB46" s="12"/>
+      <c r="AC46" s="13"/>
+      <c r="AD46" s="13"/>
+      <c r="AE46" s="13"/>
+      <c r="AF46" s="13"/>
+      <c r="AG46" s="13"/>
+      <c r="AH46" s="13"/>
+      <c r="AI46" s="14"/>
+      <c r="AJ46" s="12"/>
+      <c r="AK46" s="13"/>
+      <c r="AL46" s="13"/>
+      <c r="AM46" s="13"/>
+      <c r="AN46" s="13"/>
+      <c r="AO46" s="13"/>
+      <c r="AP46" s="13"/>
+      <c r="AQ46" s="14"/>
+      <c r="AR46" s="12"/>
+      <c r="AS46" s="13"/>
+      <c r="AT46" s="13"/>
+      <c r="AU46" s="13"/>
+      <c r="AV46" s="13"/>
+      <c r="AW46" s="13"/>
+      <c r="AX46" s="13"/>
+      <c r="AY46" s="14"/>
+      <c r="AZ46" s="12"/>
+      <c r="BA46" s="13"/>
+      <c r="BB46" s="13"/>
+      <c r="BC46" s="13"/>
+      <c r="BD46" s="13"/>
+      <c r="BE46" s="13"/>
+      <c r="BF46" s="13"/>
+      <c r="BG46" s="14"/>
+      <c r="BH46" s="12"/>
+      <c r="BI46" s="13"/>
+      <c r="BJ46" s="13"/>
+      <c r="BK46" s="13"/>
+      <c r="BL46" s="13"/>
+      <c r="BM46" s="13"/>
+      <c r="BN46" s="13"/>
+      <c r="BO46" s="14"/>
+      <c r="BP46" s="12"/>
+      <c r="BQ46" s="13"/>
+      <c r="BR46" s="13"/>
+      <c r="BS46" s="13"/>
+      <c r="BT46" s="13"/>
+      <c r="BU46" s="13"/>
+      <c r="BV46" s="13"/>
+      <c r="BW46" s="14"/>
+      <c r="BX46" s="12"/>
+      <c r="BY46" s="13"/>
+      <c r="BZ46" s="13"/>
+      <c r="CA46" s="13"/>
+      <c r="CB46" s="13"/>
+      <c r="CC46" s="13"/>
+      <c r="CD46" s="13"/>
+      <c r="CE46" s="14"/>
+      <c r="CF46" s="60"/>
+    </row>
+    <row r="47" spans="1:84" x14ac:dyDescent="0.25">
+      <c r="A47" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="B45" s="70"/>
-      <c r="C45" s="70"/>
-      <c r="D45" s="70"/>
-      <c r="E45" s="70"/>
-      <c r="F45" s="70"/>
-      <c r="G45" s="70"/>
-      <c r="H45" s="70"/>
-      <c r="I45" s="70"/>
-      <c r="J45" s="70"/>
-      <c r="K45" s="70"/>
-      <c r="L45" s="70"/>
-      <c r="M45" s="70"/>
-      <c r="N45" s="70"/>
-      <c r="O45" s="70"/>
-      <c r="P45" s="70"/>
-      <c r="Q45" s="70"/>
-      <c r="R45" s="70"/>
-      <c r="S45" s="70"/>
-      <c r="T45" s="70"/>
-      <c r="U45" s="70"/>
-      <c r="V45" s="70"/>
-      <c r="W45" s="70"/>
-      <c r="X45" s="70"/>
-      <c r="Y45" s="70"/>
-      <c r="Z45" s="70"/>
-      <c r="AA45" s="70"/>
-      <c r="AB45" s="70"/>
-      <c r="AC45" s="70"/>
-      <c r="AD45" s="70"/>
-      <c r="AE45" s="70"/>
-      <c r="AF45" s="70"/>
-      <c r="AG45" s="70"/>
-      <c r="AH45" s="70"/>
-      <c r="AI45" s="70"/>
-      <c r="AJ45" s="70"/>
-      <c r="AK45" s="70"/>
-      <c r="AL45" s="70"/>
-      <c r="AM45" s="70"/>
-      <c r="AN45" s="70"/>
-      <c r="AO45" s="70"/>
-      <c r="AP45" s="70"/>
-      <c r="AQ45" s="70"/>
-      <c r="AR45" s="70"/>
-      <c r="AS45" s="70"/>
-      <c r="AT45" s="70"/>
-      <c r="AU45" s="70"/>
-      <c r="AV45" s="70"/>
-      <c r="AW45" s="70"/>
-      <c r="AX45" s="70"/>
-      <c r="AY45" s="70"/>
-      <c r="AZ45" s="70"/>
-      <c r="BA45" s="70"/>
-      <c r="BB45" s="70"/>
-      <c r="BC45" s="70"/>
-      <c r="BD45" s="70"/>
-      <c r="BE45" s="70"/>
-      <c r="BF45" s="70"/>
-      <c r="BG45" s="70"/>
-      <c r="BH45" s="70"/>
-      <c r="BI45" s="70"/>
-      <c r="BJ45" s="70"/>
-      <c r="BK45" s="70"/>
-      <c r="BL45" s="70"/>
-      <c r="BM45" s="70"/>
-      <c r="BN45" s="70"/>
-      <c r="BO45" s="70"/>
-      <c r="BP45" s="70"/>
-      <c r="BQ45" s="70"/>
-      <c r="BR45" s="70"/>
-      <c r="BS45" s="70"/>
-      <c r="BT45" s="70"/>
-      <c r="BU45" s="70"/>
-      <c r="BV45" s="70"/>
-      <c r="BW45" s="70"/>
-      <c r="BX45" s="70"/>
-      <c r="BY45" s="70"/>
-      <c r="BZ45" s="70"/>
-      <c r="CA45" s="70"/>
-      <c r="CB45" s="70"/>
-      <c r="CC45" s="70"/>
-      <c r="CD45" s="70"/>
-      <c r="CE45" s="70"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="59"/>
+      <c r="K47" s="59"/>
+      <c r="L47" s="59"/>
+      <c r="M47" s="59"/>
+      <c r="N47" s="59"/>
+      <c r="O47" s="59"/>
+      <c r="P47" s="59"/>
+      <c r="Q47" s="59"/>
+      <c r="R47" s="59"/>
+      <c r="S47" s="59"/>
+      <c r="T47" s="59"/>
+      <c r="U47" s="59"/>
+      <c r="V47" s="59"/>
+      <c r="W47" s="59"/>
+      <c r="X47" s="59"/>
+      <c r="Y47" s="59"/>
+      <c r="Z47" s="59"/>
+      <c r="AA47" s="59"/>
+      <c r="AB47" s="59"/>
+      <c r="AC47" s="59"/>
+      <c r="AD47" s="59"/>
+      <c r="AE47" s="59"/>
+      <c r="AF47" s="59"/>
+      <c r="AG47" s="59"/>
+      <c r="AH47" s="59"/>
+      <c r="AI47" s="59"/>
+      <c r="AJ47" s="59"/>
+      <c r="AK47" s="59"/>
+      <c r="AL47" s="59"/>
+      <c r="AM47" s="59"/>
+      <c r="AN47" s="59"/>
+      <c r="AO47" s="59"/>
+      <c r="AP47" s="59"/>
+      <c r="AQ47" s="59"/>
+      <c r="AR47" s="59"/>
+      <c r="AS47" s="59"/>
+      <c r="AT47" s="59"/>
+      <c r="AU47" s="59"/>
+      <c r="AV47" s="59"/>
+      <c r="AW47" s="59"/>
+      <c r="AX47" s="59"/>
+      <c r="AY47" s="59"/>
+      <c r="AZ47" s="59"/>
+      <c r="BA47" s="59"/>
+      <c r="BB47" s="59"/>
+      <c r="BC47" s="59"/>
+      <c r="BD47" s="59"/>
+      <c r="BE47" s="59"/>
+      <c r="BF47" s="59"/>
+      <c r="BG47" s="59"/>
+      <c r="BH47" s="59"/>
+      <c r="BI47" s="59"/>
+      <c r="BJ47" s="59"/>
+      <c r="BK47" s="59"/>
+      <c r="BL47" s="59"/>
+      <c r="BM47" s="59"/>
+      <c r="BN47" s="59"/>
+      <c r="BO47" s="59"/>
+      <c r="BP47" s="59"/>
+      <c r="BQ47" s="59"/>
+      <c r="BR47" s="59"/>
+      <c r="BS47" s="59"/>
+      <c r="BT47" s="59"/>
+      <c r="BU47" s="59"/>
+      <c r="BV47" s="59"/>
+      <c r="BW47" s="59"/>
+      <c r="BX47" s="59"/>
+      <c r="BY47" s="59"/>
+      <c r="BZ47" s="59"/>
+      <c r="CA47" s="59"/>
+      <c r="CB47" s="59"/>
+      <c r="CC47" s="59"/>
+      <c r="CD47" s="59"/>
+      <c r="CE47" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A45:CE45"/>
-    <mergeCell ref="CF7:CF44"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="T9:AA44"/>
-    <mergeCell ref="AZ7:BC7"/>
-    <mergeCell ref="BD7:BG7"/>
-    <mergeCell ref="BH7:BK7"/>
-    <mergeCell ref="BL7:BO7"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="T7:W7"/>
+    <mergeCell ref="X7:AA7"/>
+    <mergeCell ref="D5:AQ6"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B4:C4"/>
     <mergeCell ref="AR5:CE6"/>
     <mergeCell ref="AJ7:AM7"/>
     <mergeCell ref="AN7:AQ7"/>
@@ -6137,17 +6412,21 @@
     <mergeCell ref="BP7:BS7"/>
     <mergeCell ref="BX7:CA7"/>
     <mergeCell ref="CB7:CE7"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="T7:W7"/>
-    <mergeCell ref="X7:AA7"/>
-    <mergeCell ref="D5:AQ6"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="A47:CE47"/>
+    <mergeCell ref="CF7:CF46"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="T9:AA46"/>
+    <mergeCell ref="AZ7:BC7"/>
+    <mergeCell ref="BD7:BG7"/>
+    <mergeCell ref="BH7:BK7"/>
+    <mergeCell ref="BL7:BO7"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
-  <conditionalFormatting sqref="B9:B44">
+  <conditionalFormatting sqref="B9:B46">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",B9)))</formula>
     </cfRule>
@@ -6386,6 +6665,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="8afaa137-8a18-4908-97f4-35fc924e5a91">
@@ -6394,15 +6682,6 @@
     <TaxCatchAll xmlns="3b60234b-33e6-42ae-ae88-ba7d4a3eedfd" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6425,6 +6704,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{762EB85F-E28B-44CA-8330-7878EE38D3E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F2702F0-3EB0-496B-8166-A9BB237AECA6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -6439,12 +6726,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{762EB85F-E28B-44CA-8330-7878EE38D3E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>